<commit_message>
Outline: house-book helper columns live on Historical Data (sample rows)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ej7a6PzaA8QN4QW543pw2j
</commit_message>
<xml_diff>
--- a/Aspire_Combined_Underwriting_Model_OUTLINE.xlsx
+++ b/Aspire_Combined_Underwriting_Model_OUTLINE.xlsx
@@ -316,7 +316,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="15">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -395,6 +395,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00EEF2FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00065F46"/>
       </patternFill>
     </fill>
   </fills>
@@ -574,7 +579,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="263">
+  <cellXfs count="267">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -1197,12 +1202,18 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="41" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="42" fillId="15" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="42" fillId="11" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="174" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="47" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="47" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="47" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="44" fillId="13" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1802,42 +1813,42 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="262" t="inlineStr">
+      <c r="A1" s="266" t="inlineStr">
         <is>
           <t>SIC2</t>
         </is>
       </c>
-      <c r="B1" s="262" t="inlineStr">
+      <c r="B1" s="266" t="inlineStr">
         <is>
           <t>Industry (SIC major group)</t>
         </is>
       </c>
-      <c r="C1" s="262" t="inlineStr">
+      <c r="C1" s="266" t="inlineStr">
         <is>
           <t>Division</t>
         </is>
       </c>
-      <c r="E1" s="262" t="inlineStr">
+      <c r="E1" s="266" t="inlineStr">
         <is>
           <t>ISO (house-book spelling, dropdown source)</t>
         </is>
       </c>
-      <c r="G1" s="262" t="inlineStr">
+      <c r="G1" s="266" t="inlineStr">
         <is>
           <t>Industry list (dropdown)</t>
         </is>
       </c>
-      <c r="I1" s="262" t="inlineStr">
+      <c r="I1" s="266" t="inlineStr">
         <is>
           <t>State</t>
         </is>
       </c>
-      <c r="K1" s="262" t="inlineStr">
+      <c r="K1" s="266" t="inlineStr">
         <is>
           <t>Fed holiday (ACH)</t>
         </is>
       </c>
-      <c r="M1" s="262" t="inlineStr">
+      <c r="M1" s="266" t="inlineStr">
         <is>
           <t>Status list</t>
         </is>
@@ -1874,7 +1885,7 @@
           <t>AL</t>
         </is>
       </c>
-      <c r="K2" s="249" t="n">
+      <c r="K2" s="250" t="n">
         <v>45292</v>
       </c>
       <c r="M2" t="inlineStr">
@@ -1914,7 +1925,7 @@
           <t>AR</t>
         </is>
       </c>
-      <c r="K3" s="249" t="n">
+      <c r="K3" s="250" t="n">
         <v>45306</v>
       </c>
       <c r="M3" t="inlineStr">
@@ -1954,7 +1965,7 @@
           <t>AZ</t>
         </is>
       </c>
-      <c r="K4" s="249" t="n">
+      <c r="K4" s="250" t="n">
         <v>45341</v>
       </c>
       <c r="M4" t="inlineStr">
@@ -1994,7 +2005,7 @@
           <t>CA</t>
         </is>
       </c>
-      <c r="K5" s="249" t="n">
+      <c r="K5" s="250" t="n">
         <v>45439</v>
       </c>
       <c r="M5" t="inlineStr">
@@ -2034,7 +2045,7 @@
           <t>CO</t>
         </is>
       </c>
-      <c r="K6" s="249" t="n">
+      <c r="K6" s="250" t="n">
         <v>45462</v>
       </c>
       <c r="M6" t="inlineStr">
@@ -2074,7 +2085,7 @@
           <t>CT</t>
         </is>
       </c>
-      <c r="K7" s="249" t="n">
+      <c r="K7" s="250" t="n">
         <v>45477</v>
       </c>
       <c r="M7" t="inlineStr">
@@ -2114,7 +2125,7 @@
           <t>DC</t>
         </is>
       </c>
-      <c r="K8" s="249" t="n">
+      <c r="K8" s="250" t="n">
         <v>45537</v>
       </c>
       <c r="M8" t="inlineStr">
@@ -2154,7 +2165,7 @@
           <t>DE</t>
         </is>
       </c>
-      <c r="K9" s="249" t="n">
+      <c r="K9" s="250" t="n">
         <v>45579</v>
       </c>
       <c r="M9" t="inlineStr">
@@ -2194,7 +2205,7 @@
           <t>FL</t>
         </is>
       </c>
-      <c r="K10" s="249" t="n">
+      <c r="K10" s="250" t="n">
         <v>45607</v>
       </c>
       <c r="M10" t="inlineStr">
@@ -2234,7 +2245,7 @@
           <t>GA</t>
         </is>
       </c>
-      <c r="K11" s="249" t="n">
+      <c r="K11" s="250" t="n">
         <v>45624</v>
       </c>
       <c r="M11" t="inlineStr">
@@ -2274,7 +2285,7 @@
           <t>HI</t>
         </is>
       </c>
-      <c r="K12" s="249" t="n">
+      <c r="K12" s="250" t="n">
         <v>45651</v>
       </c>
       <c r="M12" t="inlineStr">
@@ -2314,7 +2325,7 @@
           <t>IA</t>
         </is>
       </c>
-      <c r="K13" s="249" t="n">
+      <c r="K13" s="250" t="n">
         <v>45658</v>
       </c>
     </row>
@@ -2349,7 +2360,7 @@
           <t>ID</t>
         </is>
       </c>
-      <c r="K14" s="249" t="n">
+      <c r="K14" s="250" t="n">
         <v>45677</v>
       </c>
     </row>
@@ -2384,7 +2395,7 @@
           <t>IL</t>
         </is>
       </c>
-      <c r="K15" s="249" t="n">
+      <c r="K15" s="250" t="n">
         <v>45705</v>
       </c>
     </row>
@@ -2419,7 +2430,7 @@
           <t>IN</t>
         </is>
       </c>
-      <c r="K16" s="249" t="n">
+      <c r="K16" s="250" t="n">
         <v>45803</v>
       </c>
     </row>
@@ -2454,7 +2465,7 @@
           <t>KS</t>
         </is>
       </c>
-      <c r="K17" s="249" t="n">
+      <c r="K17" s="250" t="n">
         <v>45827</v>
       </c>
     </row>
@@ -2489,7 +2500,7 @@
           <t>KY</t>
         </is>
       </c>
-      <c r="K18" s="249" t="n">
+      <c r="K18" s="250" t="n">
         <v>45842</v>
       </c>
     </row>
@@ -2524,7 +2535,7 @@
           <t>LA</t>
         </is>
       </c>
-      <c r="K19" s="249" t="n">
+      <c r="K19" s="250" t="n">
         <v>45901</v>
       </c>
     </row>
@@ -2559,7 +2570,7 @@
           <t>MA</t>
         </is>
       </c>
-      <c r="K20" s="249" t="n">
+      <c r="K20" s="250" t="n">
         <v>45943</v>
       </c>
     </row>
@@ -2594,7 +2605,7 @@
           <t>MD</t>
         </is>
       </c>
-      <c r="K21" s="249" t="n">
+      <c r="K21" s="250" t="n">
         <v>45972</v>
       </c>
     </row>
@@ -2629,7 +2640,7 @@
           <t>ME</t>
         </is>
       </c>
-      <c r="K22" s="249" t="n">
+      <c r="K22" s="250" t="n">
         <v>45988</v>
       </c>
     </row>
@@ -2664,7 +2675,7 @@
           <t>MI</t>
         </is>
       </c>
-      <c r="K23" s="249" t="n">
+      <c r="K23" s="250" t="n">
         <v>46016</v>
       </c>
     </row>
@@ -2699,7 +2710,7 @@
           <t>MN</t>
         </is>
       </c>
-      <c r="K24" s="249" t="n">
+      <c r="K24" s="250" t="n">
         <v>46023</v>
       </c>
     </row>
@@ -2734,7 +2745,7 @@
           <t>MO</t>
         </is>
       </c>
-      <c r="K25" s="249" t="n">
+      <c r="K25" s="250" t="n">
         <v>46041</v>
       </c>
     </row>
@@ -2769,7 +2780,7 @@
           <t>MS</t>
         </is>
       </c>
-      <c r="K26" s="249" t="n">
+      <c r="K26" s="250" t="n">
         <v>46069</v>
       </c>
     </row>
@@ -2804,7 +2815,7 @@
           <t>MT</t>
         </is>
       </c>
-      <c r="K27" s="249" t="n">
+      <c r="K27" s="250" t="n">
         <v>46167</v>
       </c>
     </row>
@@ -2839,7 +2850,7 @@
           <t>NC</t>
         </is>
       </c>
-      <c r="K28" s="249" t="n">
+      <c r="K28" s="250" t="n">
         <v>46192</v>
       </c>
     </row>
@@ -2874,7 +2885,7 @@
           <t>ND</t>
         </is>
       </c>
-      <c r="K29" s="249" t="n">
+      <c r="K29" s="250" t="n">
         <v>46272</v>
       </c>
     </row>
@@ -2909,7 +2920,7 @@
           <t>NH</t>
         </is>
       </c>
-      <c r="K30" s="249" t="n">
+      <c r="K30" s="250" t="n">
         <v>46307</v>
       </c>
     </row>
@@ -2944,7 +2955,7 @@
           <t>NJ</t>
         </is>
       </c>
-      <c r="K31" s="249" t="n">
+      <c r="K31" s="250" t="n">
         <v>46337</v>
       </c>
     </row>
@@ -2979,7 +2990,7 @@
           <t>NM</t>
         </is>
       </c>
-      <c r="K32" s="249" t="n">
+      <c r="K32" s="250" t="n">
         <v>46352</v>
       </c>
     </row>
@@ -3014,7 +3025,7 @@
           <t>NV</t>
         </is>
       </c>
-      <c r="K33" s="249" t="n">
+      <c r="K33" s="250" t="n">
         <v>46381</v>
       </c>
     </row>
@@ -3049,7 +3060,7 @@
           <t>NY</t>
         </is>
       </c>
-      <c r="K34" s="249" t="n">
+      <c r="K34" s="250" t="n">
         <v>46388</v>
       </c>
     </row>
@@ -3084,7 +3095,7 @@
           <t>No state</t>
         </is>
       </c>
-      <c r="K35" s="249" t="n">
+      <c r="K35" s="250" t="n">
         <v>46405</v>
       </c>
     </row>
@@ -3119,7 +3130,7 @@
           <t>OH</t>
         </is>
       </c>
-      <c r="K36" s="249" t="n">
+      <c r="K36" s="250" t="n">
         <v>46433</v>
       </c>
     </row>
@@ -3154,7 +3165,7 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="K37" s="249" t="n">
+      <c r="K37" s="250" t="n">
         <v>46538</v>
       </c>
     </row>
@@ -3189,7 +3200,7 @@
           <t>OR</t>
         </is>
       </c>
-      <c r="K38" s="249" t="n">
+      <c r="K38" s="250" t="n">
         <v>46573</v>
       </c>
     </row>
@@ -3224,7 +3235,7 @@
           <t>PA</t>
         </is>
       </c>
-      <c r="K39" s="249" t="n">
+      <c r="K39" s="250" t="n">
         <v>46636</v>
       </c>
     </row>
@@ -3259,7 +3270,7 @@
           <t>PR</t>
         </is>
       </c>
-      <c r="K40" s="249" t="n">
+      <c r="K40" s="250" t="n">
         <v>46671</v>
       </c>
     </row>
@@ -3294,7 +3305,7 @@
           <t>RI</t>
         </is>
       </c>
-      <c r="K41" s="249" t="n">
+      <c r="K41" s="250" t="n">
         <v>46702</v>
       </c>
     </row>
@@ -3329,7 +3340,7 @@
           <t>SC</t>
         </is>
       </c>
-      <c r="K42" s="249" t="n">
+      <c r="K42" s="250" t="n">
         <v>46716</v>
       </c>
     </row>
@@ -11388,7 +11399,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BE12"/>
+  <dimension ref="A1:BR12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="230" min="1" max="1"/>
@@ -11396,39 +11407,52 @@
     <col width="22" customWidth="1" style="230" min="3" max="3"/>
     <col width="18" customWidth="1" style="230" min="4" max="4"/>
     <col width="14" customWidth="1" style="230" min="11" max="11"/>
-    <col width="16" customWidth="1" style="230" min="25" max="25"/>
-    <col width="16" customWidth="1" style="230" min="26" max="26"/>
-    <col width="16" customWidth="1" style="230" min="27" max="27"/>
-    <col width="16" customWidth="1" style="230" min="28" max="28"/>
-    <col width="16" customWidth="1" style="230" min="29" max="29"/>
-    <col width="16" customWidth="1" style="230" min="30" max="30"/>
-    <col width="16" customWidth="1" style="230" min="31" max="31"/>
-    <col width="16" customWidth="1" style="230" min="32" max="32"/>
-    <col width="16" customWidth="1" style="230" min="33" max="33"/>
-    <col width="16" customWidth="1" style="230" min="34" max="34"/>
-    <col width="16" customWidth="1" style="230" min="35" max="35"/>
-    <col width="16" customWidth="1" style="230" min="36" max="36"/>
-    <col width="16" customWidth="1" style="230" min="37" max="37"/>
-    <col width="16" customWidth="1" style="230" min="38" max="38"/>
-    <col width="16" customWidth="1" style="230" min="39" max="39"/>
-    <col width="16" customWidth="1" style="230" min="40" max="40"/>
-    <col width="16" customWidth="1" style="230" min="41" max="41"/>
-    <col width="16" customWidth="1" style="230" min="42" max="42"/>
-    <col width="16" customWidth="1" style="230" min="43" max="43"/>
-    <col width="16" customWidth="1" style="230" min="44" max="44"/>
-    <col width="16" customWidth="1" style="230" min="45" max="45"/>
-    <col width="16" customWidth="1" style="230" min="46" max="46"/>
-    <col width="16" customWidth="1" style="230" min="47" max="47"/>
-    <col width="16" customWidth="1" style="230" min="48" max="48"/>
-    <col width="16" customWidth="1" style="230" min="49" max="49"/>
-    <col width="16" customWidth="1" style="230" min="50" max="50"/>
-    <col width="16" customWidth="1" style="230" min="51" max="51"/>
-    <col width="16" customWidth="1" style="230" min="52" max="52"/>
-    <col width="16" customWidth="1" style="230" min="53" max="53"/>
-    <col width="16" customWidth="1" style="230" min="54" max="54"/>
-    <col width="16" customWidth="1" style="230" min="55" max="55"/>
-    <col width="16" customWidth="1" style="230" min="56" max="56"/>
-    <col width="16" customWidth="1" style="230" min="57" max="57"/>
+    <col width="15" customWidth="1" style="230" min="25" max="25"/>
+    <col width="15" customWidth="1" style="230" min="26" max="26"/>
+    <col width="15" customWidth="1" style="230" min="27" max="27"/>
+    <col width="15" customWidth="1" style="230" min="28" max="28"/>
+    <col width="15" customWidth="1" style="230" min="29" max="29"/>
+    <col width="15" customWidth="1" style="230" min="30" max="30"/>
+    <col width="15" customWidth="1" style="230" min="31" max="31"/>
+    <col width="15" customWidth="1" style="230" min="32" max="32"/>
+    <col width="15" customWidth="1" style="230" min="33" max="33"/>
+    <col width="15" customWidth="1" style="230" min="34" max="34"/>
+    <col width="15" customWidth="1" style="230" min="35" max="35"/>
+    <col width="15" customWidth="1" style="230" min="36" max="36"/>
+    <col width="15" customWidth="1" style="230" min="37" max="37"/>
+    <col width="15" customWidth="1" style="230" min="38" max="38"/>
+    <col width="15" customWidth="1" style="230" min="39" max="39"/>
+    <col width="15" customWidth="1" style="230" min="40" max="40"/>
+    <col width="15" customWidth="1" style="230" min="41" max="41"/>
+    <col width="15" customWidth="1" style="230" min="42" max="42"/>
+    <col width="15" customWidth="1" style="230" min="43" max="43"/>
+    <col width="15" customWidth="1" style="230" min="44" max="44"/>
+    <col width="15" customWidth="1" style="230" min="45" max="45"/>
+    <col width="15" customWidth="1" style="230" min="46" max="46"/>
+    <col width="15" customWidth="1" style="230" min="47" max="47"/>
+    <col width="15" customWidth="1" style="230" min="48" max="48"/>
+    <col width="15" customWidth="1" style="230" min="49" max="49"/>
+    <col width="15" customWidth="1" style="230" min="50" max="50"/>
+    <col width="15" customWidth="1" style="230" min="51" max="51"/>
+    <col width="15" customWidth="1" style="230" min="52" max="52"/>
+    <col width="15" customWidth="1" style="230" min="53" max="53"/>
+    <col width="15" customWidth="1" style="230" min="54" max="54"/>
+    <col width="15" customWidth="1" style="230" min="55" max="55"/>
+    <col width="15" customWidth="1" style="230" min="56" max="56"/>
+    <col width="15" customWidth="1" style="230" min="57" max="57"/>
+    <col width="15" customWidth="1" style="230" min="58" max="58"/>
+    <col width="15" customWidth="1" style="230" min="59" max="59"/>
+    <col width="15" customWidth="1" style="230" min="60" max="60"/>
+    <col width="15" customWidth="1" style="230" min="61" max="61"/>
+    <col width="15" customWidth="1" style="230" min="62" max="62"/>
+    <col width="15" customWidth="1" style="230" min="63" max="63"/>
+    <col width="15" customWidth="1" style="230" min="64" max="64"/>
+    <col width="15" customWidth="1" style="230" min="65" max="65"/>
+    <col width="15" customWidth="1" style="230" min="66" max="66"/>
+    <col width="15" customWidth="1" style="230" min="67" max="67"/>
+    <col width="15" customWidth="1" style="230" min="68" max="68"/>
+    <col width="15" customWidth="1" style="230" min="69" max="69"/>
+    <col width="15" customWidth="1" style="230" min="70" max="70"/>
   </cols>
   <sheetData>
     <row r="1" ht="42" customHeight="1" s="230">
@@ -11554,165 +11578,230 @@
       </c>
       <c r="Y1" s="248" t="inlineStr">
         <is>
+          <t>Unit of raw duration</t>
+        </is>
+      </c>
+      <c r="Z1" s="248" t="inlineStr">
+        <is>
+          <t>Pay frequency</t>
+        </is>
+      </c>
+      <c r="AA1" s="248" t="inlineStr">
+        <is>
+          <t>Expected term (payments)</t>
+        </is>
+      </c>
+      <c r="AB1" s="248" t="inlineStr">
+        <is>
+          <t>Expected term (business days)</t>
+        </is>
+      </c>
+      <c r="AC1" s="248" t="inlineStr">
+        <is>
+          <t>Actual days on book (calendar)</t>
+        </is>
+      </c>
+      <c r="AD1" s="248" t="inlineStr">
+        <is>
+          <t>Actual days on book (business)</t>
+        </is>
+      </c>
+      <c r="AE1" s="248" t="inlineStr">
+        <is>
+          <t>Default</t>
+        </is>
+      </c>
+      <c r="AF1" s="248" t="inlineStr">
+        <is>
+          <t>Resolved</t>
+        </is>
+      </c>
+      <c r="AG1" s="248" t="inlineStr">
+        <is>
+          <t>Closed family</t>
+        </is>
+      </c>
+      <c r="AH1" s="248" t="inlineStr">
+        <is>
+          <t>In scope</t>
+        </is>
+      </c>
+      <c r="AI1" s="248" t="inlineStr">
+        <is>
+          <t>Net cash</t>
+        </is>
+      </c>
+      <c r="AJ1" s="248" t="inlineStr">
+        <is>
+          <t>Principal lost</t>
+        </is>
+      </c>
+      <c r="AK1" s="248" t="inlineStr">
+        <is>
+          <t>Collected %</t>
+        </is>
+      </c>
+      <c r="AL1" s="248" t="inlineStr">
+        <is>
+          <t>Advance / revenue</t>
+        </is>
+      </c>
+      <c r="AM1" s="248" t="inlineStr">
+        <is>
+          <t>Has revenue</t>
+        </is>
+      </c>
+      <c r="AN1" s="248" t="inlineStr">
+        <is>
+          <t>Never paid</t>
+        </is>
+      </c>
+      <c r="AO1" s="248" t="inlineStr">
+        <is>
+          <t>Days on book (defaulted deals)</t>
+        </is>
+      </c>
+      <c r="AP1" s="248" t="inlineStr">
+        <is>
+          <t>Days to close</t>
+        </is>
+      </c>
+      <c r="AQ1" s="248" t="inlineStr">
+        <is>
+          <t>Size bucket</t>
+        </is>
+      </c>
+      <c r="AR1" s="248" t="inlineStr">
+        <is>
+          <t>Factor bucket</t>
+        </is>
+      </c>
+      <c r="AS1" s="248" t="inlineStr">
+        <is>
+          <t>Term bucket</t>
+        </is>
+      </c>
+      <c r="AT1" s="248" t="inlineStr">
+        <is>
+          <t>Adv/rev bucket</t>
+        </is>
+      </c>
+      <c r="AU1" s="248" t="inlineStr">
+        <is>
           <t>Industry</t>
         </is>
       </c>
-      <c r="Z1" s="248" t="inlineStr">
-        <is>
-          <t>Pay frequency</t>
-        </is>
-      </c>
-      <c r="AA1" s="248" t="inlineStr">
-        <is>
-          <t>Term (bus. days)</t>
-        </is>
-      </c>
-      <c r="AB1" s="248" t="inlineStr">
+      <c r="AV1" s="248" t="inlineStr">
+        <is>
+          <t>Quarter</t>
+        </is>
+      </c>
+      <c r="AW1" s="248" t="inlineStr">
+        <is>
+          <t>Month</t>
+        </is>
+      </c>
+      <c r="AX1" s="248" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="AY1" s="249" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="AZ1" s="249" t="inlineStr">
         <is>
           <t>Age at as-of (bus. days)</t>
         </is>
       </c>
-      <c r="AC1" s="248" t="inlineStr">
+      <c r="BA1" s="249" t="inlineStr">
         <is>
           <t>Seasoned</t>
         </is>
       </c>
-      <c r="AD1" s="248" t="inlineStr">
-        <is>
-          <t>In window</t>
-        </is>
-      </c>
-      <c r="AE1" s="248" t="inlineStr">
-        <is>
-          <t>Default</t>
-        </is>
-      </c>
-      <c r="AF1" s="248" t="inlineStr">
-        <is>
-          <t>Resolved</t>
-        </is>
-      </c>
-      <c r="AG1" s="248" t="inlineStr">
-        <is>
-          <t>Closed family</t>
-        </is>
-      </c>
-      <c r="AH1" s="248" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="AI1" s="248" t="inlineStr">
-        <is>
-          <t>Status valid</t>
-        </is>
-      </c>
-      <c r="AJ1" s="248" t="inlineStr">
-        <is>
-          <t>Net cash</t>
-        </is>
-      </c>
-      <c r="AK1" s="248" t="inlineStr">
-        <is>
-          <t>Principal lost</t>
-        </is>
-      </c>
-      <c r="AL1" s="248" t="inlineStr">
-        <is>
-          <t>Adv / revenue</t>
-        </is>
-      </c>
-      <c r="AM1" s="248" t="inlineStr">
-        <is>
-          <t>Has revenue</t>
-        </is>
-      </c>
-      <c r="AN1" s="248" t="inlineStr">
-        <is>
-          <t>Days on book (bus.)</t>
-        </is>
-      </c>
-      <c r="AO1" s="248" t="inlineStr">
+      <c r="BB1" s="249" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
+      <c r="BC1" s="249" t="inlineStr">
         <is>
           <t>Renewal</t>
         </is>
       </c>
-      <c r="AP1" s="248" t="inlineStr">
-        <is>
-          <t>Eligible</t>
-        </is>
-      </c>
-      <c r="AQ1" s="248" t="inlineStr">
+      <c r="BD1" s="249" t="inlineStr">
         <is>
           <t>m: position</t>
         </is>
       </c>
-      <c r="AR1" s="248" t="inlineStr">
+      <c r="BE1" s="249" t="inlineStr">
         <is>
           <t>m: new/renewal</t>
         </is>
       </c>
-      <c r="AS1" s="248" t="inlineStr">
+      <c r="BF1" s="249" t="inlineStr">
         <is>
           <t>m: industry</t>
         </is>
       </c>
-      <c r="AT1" s="248" t="inlineStr">
+      <c r="BG1" s="249" t="inlineStr">
         <is>
           <t>m: ISO</t>
         </is>
       </c>
-      <c r="AU1" s="248" t="inlineStr">
+      <c r="BH1" s="249" t="inlineStr">
         <is>
           <t>m: state</t>
         </is>
       </c>
-      <c r="AV1" s="248" t="inlineStr">
+      <c r="BI1" s="249" t="inlineStr">
         <is>
           <t>T1 NR+Ind+Pos</t>
         </is>
       </c>
-      <c r="AW1" s="248" t="inlineStr">
+      <c r="BJ1" s="249" t="inlineStr">
         <is>
           <t>T2 NR+ISO+Pos</t>
         </is>
       </c>
-      <c r="AX1" s="248" t="inlineStr">
+      <c r="BK1" s="249" t="inlineStr">
         <is>
           <t>T3 NR+Ind</t>
         </is>
       </c>
-      <c r="AY1" s="248" t="inlineStr">
+      <c r="BL1" s="249" t="inlineStr">
         <is>
           <t>T4 NR+ISO</t>
         </is>
       </c>
-      <c r="AZ1" s="248" t="inlineStr">
+      <c r="BM1" s="249" t="inlineStr">
         <is>
           <t>T5 NR+Pos</t>
         </is>
       </c>
-      <c r="BA1" s="248" t="inlineStr">
+      <c r="BN1" s="249" t="inlineStr">
         <is>
           <t>T6 NR</t>
         </is>
       </c>
-      <c r="BB1" s="248" t="inlineStr">
+      <c r="BO1" s="249" t="inlineStr">
         <is>
           <t>T7 Book</t>
         </is>
       </c>
-      <c r="BC1" s="248" t="inlineStr">
+      <c r="BP1" s="249" t="inlineStr">
         <is>
           <t>Best tier</t>
         </is>
       </c>
-      <c r="BD1" s="248" t="inlineStr">
+      <c r="BQ1" s="249" t="inlineStr">
         <is>
           <t>In primary cohort</t>
         </is>
       </c>
-      <c r="BE1" s="248" t="inlineStr">
+      <c r="BR1" s="249" t="inlineStr">
         <is>
           <t>Seq</t>
         </is>
@@ -11724,167 +11813,232 @@
           <t>RAW from CRM export (values) →</t>
         </is>
       </c>
-      <c r="Y2" s="242" t="inlineStr">
-        <is>
-          <t>→ SIC2 looked up on Ref (blank -&gt; "No SIC")</t>
-        </is>
-      </c>
-      <c r="Z2" s="242" t="inlineStr">
-        <is>
-          <t>→ raw duration &lt; 12 = months = Daily deal; &gt;= 12 = weeks = Weekly deal</t>
-        </is>
-      </c>
-      <c r="AA2" s="242" t="inlineStr">
-        <is>
-          <t>→ months x 21.655 or weeks x 5</t>
-        </is>
-      </c>
-      <c r="AB2" s="242" t="inlineStr">
+      <c r="Y2" s="236" t="inlineStr">
+        <is>
+          <t>LIVE (house book): raw &lt; 12 = Months (daily deal), &gt;= 12 = Weeks (weekly deal)</t>
+        </is>
+      </c>
+      <c r="Z2" s="236" t="inlineStr">
+        <is>
+          <t>LIVE (house book): Months -&gt; Daily, Weeks -&gt; Weekly</t>
+        </is>
+      </c>
+      <c r="AA2" s="236" t="inlineStr">
+        <is>
+          <t>LIVE (house book): months x 21.655, or weeks</t>
+        </is>
+      </c>
+      <c r="AB2" s="236" t="inlineStr">
+        <is>
+          <t>LIVE (house book): months x 21.655, or weeks x 5</t>
+        </is>
+      </c>
+      <c r="AC2" s="236" t="inlineStr">
+        <is>
+          <t>LIVE (house book): last active - funding</t>
+        </is>
+      </c>
+      <c r="AD2" s="236" t="inlineStr">
+        <is>
+          <t>LIVE (house book): NETWORKDAYS(funding, last active, Fed holidays)</t>
+        </is>
+      </c>
+      <c r="AE2" s="236" t="inlineStr">
+        <is>
+          <t>LIVE (house book): status mapping, col 2</t>
+        </is>
+      </c>
+      <c r="AF2" s="236" t="inlineStr">
+        <is>
+          <t>LIVE (house book): status mapping, col 3</t>
+        </is>
+      </c>
+      <c r="AG2" s="236" t="inlineStr">
+        <is>
+          <t>LIVE (house book): status mapping, col 4</t>
+        </is>
+      </c>
+      <c r="AH2" s="236" t="inlineStr">
+        <is>
+          <t>LIVE (house book): funded inside the Controls window</t>
+        </is>
+      </c>
+      <c r="AI2" s="236" t="inlineStr">
+        <is>
+          <t>LIVE (house book): collected - advance</t>
+        </is>
+      </c>
+      <c r="AJ2" s="236" t="inlineStr">
+        <is>
+          <t>LIVE (house book): MAX(advance - collected, 0) on defaulted deals</t>
+        </is>
+      </c>
+      <c r="AK2" s="236" t="inlineStr">
+        <is>
+          <t>LIVE (house book): collected / advance</t>
+        </is>
+      </c>
+      <c r="AL2" s="236" t="inlineStr">
+        <is>
+          <t>LIVE (house book): advance / avg monthly revenue; blank when missing</t>
+        </is>
+      </c>
+      <c r="AM2" s="236" t="inlineStr">
+        <is>
+          <t>LIVE (house book): 1 if revenue present</t>
+        </is>
+      </c>
+      <c r="AN2" s="236" t="inlineStr">
+        <is>
+          <t>LIVE (house book): 1 if collected &lt;= 0</t>
+        </is>
+      </c>
+      <c r="AO2" s="236" t="inlineStr">
+        <is>
+          <t>LIVE (house book): business days, defaulted only</t>
+        </is>
+      </c>
+      <c r="AP2" s="236" t="inlineStr">
+        <is>
+          <t>LIVE (house book): business days, non-defaulted Closed family</t>
+        </is>
+      </c>
+      <c r="AQ2" s="236" t="inlineStr">
+        <is>
+          <t>LIVE (house book): six advance buckets</t>
+        </is>
+      </c>
+      <c r="AR2" s="236" t="inlineStr">
+        <is>
+          <t>LIVE (house book): six factor buckets</t>
+        </is>
+      </c>
+      <c r="AS2" s="236" t="inlineStr">
+        <is>
+          <t>LIVE (house book): cut on business days</t>
+        </is>
+      </c>
+      <c r="AT2" s="236" t="inlineStr">
+        <is>
+          <t>LIVE (house book): with a "No revenue data" bucket</t>
+        </is>
+      </c>
+      <c r="AU2" s="236" t="inlineStr">
+        <is>
+          <t>LIVE (house book): SIC2 looked up on Ref</t>
+        </is>
+      </c>
+      <c r="AV2" s="236" t="inlineStr">
+        <is>
+          <t>LIVE (house book): funding quarter</t>
+        </is>
+      </c>
+      <c r="AW2" s="236" t="inlineStr">
+        <is>
+          <t>LIVE (house book): funding month</t>
+        </is>
+      </c>
+      <c r="AX2" s="236" t="inlineStr">
+        <is>
+          <t>LIVE (house book): funding year</t>
+        </is>
+      </c>
+      <c r="AY2" s="242" t="inlineStr">
+        <is>
+          <t>→ from status mapping col 5 (new column in the mapping)</t>
+        </is>
+      </c>
+      <c r="AZ2" s="242" t="inlineStr">
         <is>
           <t>→ NETWORKDAYS(funding date, Controls as-of date, holidays)</t>
         </is>
       </c>
-      <c r="AC2" s="242" t="inlineStr">
-        <is>
-          <t>→ 1 if age &gt;= seasoning multiple x term</t>
-        </is>
-      </c>
-      <c r="AD2" s="242" t="inlineStr">
-        <is>
-          <t>→ 1 if funded inside the Controls window</t>
-        </is>
-      </c>
-      <c r="AE2" s="242" t="inlineStr">
-        <is>
-          <t>→ from status mapping</t>
-        </is>
-      </c>
-      <c r="AF2" s="242" t="inlineStr">
-        <is>
-          <t>→ from status mapping</t>
-        </is>
-      </c>
-      <c r="AG2" s="242" t="inlineStr">
-        <is>
-          <t>→ from status mapping</t>
-        </is>
-      </c>
-      <c r="AH2" s="242" t="inlineStr">
-        <is>
-          <t>→ from status mapping</t>
-        </is>
-      </c>
-      <c r="AI2" s="242" t="inlineStr">
-        <is>
-          <t>→ 1 if status is in the mapping table</t>
-        </is>
-      </c>
-      <c r="AJ2" s="242" t="inlineStr">
-        <is>
-          <t>→ collected - advance</t>
-        </is>
-      </c>
-      <c r="AK2" s="242" t="inlineStr">
-        <is>
-          <t>→ MAX(advance - collected, 0) on defaulted deals, else 0</t>
-        </is>
-      </c>
-      <c r="AL2" s="242" t="inlineStr">
-        <is>
-          <t>→ advance / avg monthly revenue (0 + "has revenue" flag when missing)</t>
-        </is>
-      </c>
-      <c r="AM2" s="242" t="inlineStr">
-        <is>
-          <t>→ 1 if revenue present</t>
-        </is>
-      </c>
-      <c r="AN2" s="242" t="inlineStr">
-        <is>
-          <t>→ NETWORKDAYS(funding, last active)</t>
-        </is>
-      </c>
-      <c r="AO2" s="242" t="inlineStr">
+      <c r="BA2" s="242" t="inlineStr">
+        <is>
+          <t>→ 1 if age &gt;= seasoning multiple x expected term (business days)</t>
+        </is>
+      </c>
+      <c r="BB2" s="242" t="inlineStr">
+        <is>
+          <t>→ seasoned x in-scope: the only rows that enter a rate</t>
+        </is>
+      </c>
+      <c r="BC2" s="242" t="inlineStr">
         <is>
           <t>→ 1 if Renewal</t>
         </is>
       </c>
-      <c r="AP2" s="242" t="inlineStr">
-        <is>
-          <t>→ seasoned x in-window: the only rows that enter a rate</t>
-        </is>
-      </c>
-      <c r="AQ2" s="242" t="inlineStr">
+      <c r="BD2" s="242" t="inlineStr">
         <is>
           <t>→ 1 if position = proposed position on Deal</t>
         </is>
       </c>
-      <c r="AR2" s="242" t="inlineStr">
+      <c r="BE2" s="242" t="inlineStr">
         <is>
           <t>→ 1 if same as Deal</t>
         </is>
       </c>
-      <c r="AS2" s="242" t="inlineStr">
+      <c r="BF2" s="242" t="inlineStr">
         <is>
           <t>→ 1 if same as Deal</t>
         </is>
       </c>
-      <c r="AT2" s="242" t="inlineStr">
+      <c r="BG2" s="242" t="inlineStr">
         <is>
           <t>→ 1 if same as Deal</t>
         </is>
       </c>
-      <c r="AU2" s="242" t="inlineStr">
+      <c r="BH2" s="242" t="inlineStr">
         <is>
           <t>→ 1 if same as Deal</t>
         </is>
       </c>
-      <c r="AV2" s="242" t="inlineStr">
+      <c r="BI2" s="242" t="inlineStr">
         <is>
           <t>→ m:NR x m:Ind x m:Pos</t>
         </is>
       </c>
-      <c r="AW2" s="242" t="inlineStr">
+      <c r="BJ2" s="242" t="inlineStr">
         <is>
           <t>→ m:NR x m:ISO x m:Pos</t>
         </is>
       </c>
-      <c r="AX2" s="242" t="inlineStr">
+      <c r="BK2" s="242" t="inlineStr">
         <is>
           <t>→ m:NR x m:Ind</t>
         </is>
       </c>
-      <c r="AY2" s="242" t="inlineStr">
+      <c r="BL2" s="242" t="inlineStr">
         <is>
           <t>→ m:NR x m:ISO</t>
         </is>
       </c>
-      <c r="AZ2" s="242" t="inlineStr">
+      <c r="BM2" s="242" t="inlineStr">
         <is>
           <t>→ m:NR x m:Pos</t>
         </is>
       </c>
-      <c r="BA2" s="242" t="inlineStr">
+      <c r="BN2" s="242" t="inlineStr">
         <is>
           <t>→ m:NR</t>
         </is>
       </c>
-      <c r="BB2" s="242" t="inlineStr">
+      <c r="BO2" s="242" t="inlineStr">
         <is>
           <t>→ always 1</t>
         </is>
       </c>
-      <c r="BC2" s="242" t="inlineStr">
+      <c r="BP2" s="242" t="inlineStr">
         <is>
           <t>→ lowest tier number the deal matches</t>
         </is>
       </c>
-      <c r="BD2" s="242" t="inlineStr">
+      <c r="BQ2" s="242" t="inlineStr">
         <is>
           <t>→ 1 if the deal matches the primary tier chosen on Historical Score</t>
         </is>
       </c>
-      <c r="BE2" s="242" t="inlineStr">
+      <c r="BR2" s="242" t="inlineStr">
         <is>
           <t>→ running count of in-primary-cohort rows; feeds the Comparable Deals list</t>
         </is>
@@ -11911,10 +12065,10 @@
           <t>Closed</t>
         </is>
       </c>
-      <c r="E3" s="249" t="n">
+      <c r="E3" s="250" t="n">
         <v>45672</v>
       </c>
-      <c r="F3" s="249" t="n">
+      <c r="F3" s="250" t="n">
         <v>45821</v>
       </c>
       <c r="G3" t="n">
@@ -11948,22 +12102,22 @@
       <c r="M3" t="n">
         <v>1.5</v>
       </c>
-      <c r="N3" s="250" t="n">
+      <c r="N3" s="251" t="n">
         <v>10000</v>
       </c>
-      <c r="O3" s="250" t="n">
+      <c r="O3" s="251" t="n">
         <v>1000</v>
       </c>
-      <c r="P3" s="250" t="n">
+      <c r="P3" s="251" t="n">
         <v>15000</v>
       </c>
-      <c r="Q3" s="250" t="n">
+      <c r="Q3" s="251" t="n">
         <v>15000</v>
       </c>
-      <c r="R3" s="250" t="n">
+      <c r="R3" s="251" t="n">
         <v>0</v>
       </c>
-      <c r="S3" s="251" t="n">
+      <c r="S3" s="252" t="n">
         <v>1</v>
       </c>
       <c r="T3" t="n">
@@ -11975,11 +12129,115 @@
       <c r="V3" t="n">
         <v>50000</v>
       </c>
-      <c r="W3" s="251" t="n">
+      <c r="W3" s="252" t="n">
         <v>0.12</v>
       </c>
-      <c r="X3" s="249" t="n">
+      <c r="X3" s="250" t="n">
         <v>43160</v>
+      </c>
+      <c r="Y3" s="253">
+        <f>IF(T3="","",IF(T3&lt;12,"Months","Weeks"))</f>
+        <v/>
+      </c>
+      <c r="Z3" s="253">
+        <f>IF(Y3="","",IF(Y3="Months","Daily","Weekly"))</f>
+        <v/>
+      </c>
+      <c r="AA3" s="253">
+        <f>IF(T3="","",IF(Z3="Daily",T3*Controls!$B$29,T3))</f>
+        <v/>
+      </c>
+      <c r="AB3" s="253">
+        <f>IF(T3="","",IF(Z3="Daily",T3*Controls!$B$29,T3*5))</f>
+        <v/>
+      </c>
+      <c r="AC3" s="253">
+        <f>IF(OR(E3="",F3=""),"",F3-E3)</f>
+        <v/>
+      </c>
+      <c r="AD3" s="253">
+        <f>IF(OR(E3="",F3=""),"",NETWORKDAYS(E3,F3,Ref!$K$2:$K$42))</f>
+        <v/>
+      </c>
+      <c r="AE3" s="253">
+        <f>IF(IFERROR(VLOOKUP(D3,Controls!$A$61:$E$71,2,FALSE),"No")="Yes",1,0)</f>
+        <v/>
+      </c>
+      <c r="AF3" s="253">
+        <f>IF(IFERROR(VLOOKUP(D3,Controls!$A$61:$E$71,3,FALSE),"No")="Yes",1,0)</f>
+        <v/>
+      </c>
+      <c r="AG3" s="253">
+        <f>IF(IFERROR(VLOOKUP(D3,Controls!$A$61:$E$71,4,FALSE),"No")="Yes",1,0)</f>
+        <v/>
+      </c>
+      <c r="AH3" s="253">
+        <f>IF(AND(E3&lt;&gt;"",E3&gt;=Controls!$B$37,E3&lt;=Controls!$B$38),1,0)</f>
+        <v/>
+      </c>
+      <c r="AI3" s="254">
+        <f>Q3-N3</f>
+        <v/>
+      </c>
+      <c r="AJ3" s="254">
+        <f>IF(AE3=1,MAX(0,N3-Q3),0)</f>
+        <v/>
+      </c>
+      <c r="AK3" s="255">
+        <f>IFERROR(Q3/N3,"")</f>
+        <v/>
+      </c>
+      <c r="AL3" s="255">
+        <f>IF(V3="","",N3/V3)</f>
+        <v/>
+      </c>
+      <c r="AM3" s="253">
+        <f>IF(V3="",0,1)</f>
+        <v/>
+      </c>
+      <c r="AN3" s="253">
+        <f>IF(Q3&lt;=0,1,0)</f>
+        <v/>
+      </c>
+      <c r="AO3" s="253">
+        <f>IF(AE3=1,AD3,"")</f>
+        <v/>
+      </c>
+      <c r="AP3" s="253">
+        <f>IF(AND(AE3=0,AG3=1),AD3,"")</f>
+        <v/>
+      </c>
+      <c r="AQ3" s="253">
+        <f>IF(N3&lt;10000,"Under $10K",IF(N3&lt;20000,"$10-20K",IF(N3&lt;30000,"$20-30K",IF(N3&lt;50000,"$30-50K",IF(N3&lt;100000,"$50-100K","$100K+")))))</f>
+        <v/>
+      </c>
+      <c r="AR3" s="253">
+        <f>IF(M3&lt;=1.35,"1.35 and under",IF(M3&lt;=1.42,"1.36-1.42",IF(M3&lt;=1.45,"1.43-1.45",IF(M3&lt;1.49,"1.46-1.48",IF(M3&lt;=1.49,"1.49","Above 1.49")))))</f>
+        <v/>
+      </c>
+      <c r="AS3" s="253">
+        <f>IF(AB3="","",IF(AB3&lt;60,"Under 60",IF(AB3&lt;90,"60-89",IF(AB3&lt;120,"90-119",IF(AB3&lt;150,"120-149","150+")))))</f>
+        <v/>
+      </c>
+      <c r="AT3" s="253">
+        <f>IF(AL3="","No revenue data",IF(AL3&lt;0.15,"Under 0.15x",IF(AL3&lt;0.3,"0.15-0.30x",IF(AL3&lt;0.5,"0.30-0.50x",IF(AL3&lt;1,"0.50-1.00x","1.00x+")))))</f>
+        <v/>
+      </c>
+      <c r="AU3" s="253">
+        <f>IF(I3="","No SIC",IFERROR(VLOOKUP(I3,Ref!$A$2:$B$65,2,FALSE),"Unclassified"))</f>
+        <v/>
+      </c>
+      <c r="AV3" s="253">
+        <f>IF(E3="","",TEXT(E3,"YYYY")&amp;"-Q"&amp;ROUNDUP(MONTH(E3)/3,0))</f>
+        <v/>
+      </c>
+      <c r="AW3" s="253">
+        <f>IF(E3="","",TEXT(E3,"YYYY-MM"))</f>
+        <v/>
+      </c>
+      <c r="AX3" s="253">
+        <f>IF(E3="","",TEXT(E3,"YYYY"))</f>
+        <v/>
       </c>
     </row>
     <row r="4">
@@ -12003,10 +12261,10 @@
           <t>Closed</t>
         </is>
       </c>
-      <c r="E4" s="249" t="n">
+      <c r="E4" s="250" t="n">
         <v>45698</v>
       </c>
-      <c r="F4" s="249" t="n">
+      <c r="F4" s="250" t="n">
         <v>45848</v>
       </c>
       <c r="G4" t="n">
@@ -12040,22 +12298,22 @@
       <c r="M4" t="n">
         <v>1.5</v>
       </c>
-      <c r="N4" s="250" t="n">
+      <c r="N4" s="251" t="n">
         <v>20000</v>
       </c>
-      <c r="O4" s="250" t="n">
+      <c r="O4" s="251" t="n">
         <v>2000</v>
       </c>
-      <c r="P4" s="250" t="n">
+      <c r="P4" s="251" t="n">
         <v>30000</v>
       </c>
-      <c r="Q4" s="250" t="n">
+      <c r="Q4" s="251" t="n">
         <v>30000</v>
       </c>
-      <c r="R4" s="250" t="n">
+      <c r="R4" s="251" t="n">
         <v>0</v>
       </c>
-      <c r="S4" s="251" t="n">
+      <c r="S4" s="252" t="n">
         <v>1</v>
       </c>
       <c r="T4" t="n">
@@ -12067,11 +12325,115 @@
       <c r="V4" t="n">
         <v>100000</v>
       </c>
-      <c r="W4" s="251" t="n">
+      <c r="W4" s="252" t="n">
         <v>0.09</v>
       </c>
-      <c r="X4" s="249" t="n">
+      <c r="X4" s="250" t="n">
         <v>42170</v>
+      </c>
+      <c r="Y4" s="253">
+        <f>IF(T4="","",IF(T4&lt;12,"Months","Weeks"))</f>
+        <v/>
+      </c>
+      <c r="Z4" s="253">
+        <f>IF(Y4="","",IF(Y4="Months","Daily","Weekly"))</f>
+        <v/>
+      </c>
+      <c r="AA4" s="253">
+        <f>IF(T4="","",IF(Z4="Daily",T4*Controls!$B$29,T4))</f>
+        <v/>
+      </c>
+      <c r="AB4" s="253">
+        <f>IF(T4="","",IF(Z4="Daily",T4*Controls!$B$29,T4*5))</f>
+        <v/>
+      </c>
+      <c r="AC4" s="253">
+        <f>IF(OR(E4="",F4=""),"",F4-E4)</f>
+        <v/>
+      </c>
+      <c r="AD4" s="253">
+        <f>IF(OR(E4="",F4=""),"",NETWORKDAYS(E4,F4,Ref!$K$2:$K$42))</f>
+        <v/>
+      </c>
+      <c r="AE4" s="253">
+        <f>IF(IFERROR(VLOOKUP(D4,Controls!$A$61:$E$71,2,FALSE),"No")="Yes",1,0)</f>
+        <v/>
+      </c>
+      <c r="AF4" s="253">
+        <f>IF(IFERROR(VLOOKUP(D4,Controls!$A$61:$E$71,3,FALSE),"No")="Yes",1,0)</f>
+        <v/>
+      </c>
+      <c r="AG4" s="253">
+        <f>IF(IFERROR(VLOOKUP(D4,Controls!$A$61:$E$71,4,FALSE),"No")="Yes",1,0)</f>
+        <v/>
+      </c>
+      <c r="AH4" s="253">
+        <f>IF(AND(E4&lt;&gt;"",E4&gt;=Controls!$B$37,E4&lt;=Controls!$B$38),1,0)</f>
+        <v/>
+      </c>
+      <c r="AI4" s="254">
+        <f>Q4-N4</f>
+        <v/>
+      </c>
+      <c r="AJ4" s="254">
+        <f>IF(AE4=1,MAX(0,N4-Q4),0)</f>
+        <v/>
+      </c>
+      <c r="AK4" s="255">
+        <f>IFERROR(Q4/N4,"")</f>
+        <v/>
+      </c>
+      <c r="AL4" s="255">
+        <f>IF(V4="","",N4/V4)</f>
+        <v/>
+      </c>
+      <c r="AM4" s="253">
+        <f>IF(V4="",0,1)</f>
+        <v/>
+      </c>
+      <c r="AN4" s="253">
+        <f>IF(Q4&lt;=0,1,0)</f>
+        <v/>
+      </c>
+      <c r="AO4" s="253">
+        <f>IF(AE4=1,AD4,"")</f>
+        <v/>
+      </c>
+      <c r="AP4" s="253">
+        <f>IF(AND(AE4=0,AG4=1),AD4,"")</f>
+        <v/>
+      </c>
+      <c r="AQ4" s="253">
+        <f>IF(N4&lt;10000,"Under $10K",IF(N4&lt;20000,"$10-20K",IF(N4&lt;30000,"$20-30K",IF(N4&lt;50000,"$30-50K",IF(N4&lt;100000,"$50-100K","$100K+")))))</f>
+        <v/>
+      </c>
+      <c r="AR4" s="253">
+        <f>IF(M4&lt;=1.35,"1.35 and under",IF(M4&lt;=1.42,"1.36-1.42",IF(M4&lt;=1.45,"1.43-1.45",IF(M4&lt;1.49,"1.46-1.48",IF(M4&lt;=1.49,"1.49","Above 1.49")))))</f>
+        <v/>
+      </c>
+      <c r="AS4" s="253">
+        <f>IF(AB4="","",IF(AB4&lt;60,"Under 60",IF(AB4&lt;90,"60-89",IF(AB4&lt;120,"90-119",IF(AB4&lt;150,"120-149","150+")))))</f>
+        <v/>
+      </c>
+      <c r="AT4" s="253">
+        <f>IF(AL4="","No revenue data",IF(AL4&lt;0.15,"Under 0.15x",IF(AL4&lt;0.3,"0.15-0.30x",IF(AL4&lt;0.5,"0.30-0.50x",IF(AL4&lt;1,"0.50-1.00x","1.00x+")))))</f>
+        <v/>
+      </c>
+      <c r="AU4" s="253">
+        <f>IF(I4="","No SIC",IFERROR(VLOOKUP(I4,Ref!$A$2:$B$65,2,FALSE),"Unclassified"))</f>
+        <v/>
+      </c>
+      <c r="AV4" s="253">
+        <f>IF(E4="","",TEXT(E4,"YYYY")&amp;"-Q"&amp;ROUNDUP(MONTH(E4)/3,0))</f>
+        <v/>
+      </c>
+      <c r="AW4" s="253">
+        <f>IF(E4="","",TEXT(E4,"YYYY-MM"))</f>
+        <v/>
+      </c>
+      <c r="AX4" s="253">
+        <f>IF(E4="","",TEXT(E4,"YYYY"))</f>
+        <v/>
       </c>
     </row>
     <row r="5">
@@ -12095,10 +12457,10 @@
           <t>Legal</t>
         </is>
       </c>
-      <c r="E5" s="249" t="n">
+      <c r="E5" s="250" t="n">
         <v>45721</v>
       </c>
-      <c r="F5" s="249" t="n">
+      <c r="F5" s="250" t="n">
         <v>45813</v>
       </c>
       <c r="G5" t="n">
@@ -12132,22 +12494,22 @@
       <c r="M5" t="n">
         <v>1.5</v>
       </c>
-      <c r="N5" s="250" t="n">
+      <c r="N5" s="251" t="n">
         <v>30000</v>
       </c>
-      <c r="O5" s="250" t="n">
+      <c r="O5" s="251" t="n">
         <v>3000</v>
       </c>
-      <c r="P5" s="250" t="n">
+      <c r="P5" s="251" t="n">
         <v>45000</v>
       </c>
-      <c r="Q5" s="250" t="n">
+      <c r="Q5" s="251" t="n">
         <v>9000</v>
       </c>
-      <c r="R5" s="250" t="n">
+      <c r="R5" s="251" t="n">
         <v>36000</v>
       </c>
-      <c r="S5" s="251" t="n">
+      <c r="S5" s="252" t="n">
         <v>0.2</v>
       </c>
       <c r="T5" t="n">
@@ -12159,11 +12521,115 @@
       <c r="V5" t="n">
         <v>60000</v>
       </c>
-      <c r="W5" s="251" t="n">
+      <c r="W5" s="252" t="n">
         <v>0.15</v>
       </c>
-      <c r="X5" s="249" t="n">
+      <c r="X5" s="250" t="n">
         <v>43840</v>
+      </c>
+      <c r="Y5" s="253">
+        <f>IF(T5="","",IF(T5&lt;12,"Months","Weeks"))</f>
+        <v/>
+      </c>
+      <c r="Z5" s="253">
+        <f>IF(Y5="","",IF(Y5="Months","Daily","Weekly"))</f>
+        <v/>
+      </c>
+      <c r="AA5" s="253">
+        <f>IF(T5="","",IF(Z5="Daily",T5*Controls!$B$29,T5))</f>
+        <v/>
+      </c>
+      <c r="AB5" s="253">
+        <f>IF(T5="","",IF(Z5="Daily",T5*Controls!$B$29,T5*5))</f>
+        <v/>
+      </c>
+      <c r="AC5" s="253">
+        <f>IF(OR(E5="",F5=""),"",F5-E5)</f>
+        <v/>
+      </c>
+      <c r="AD5" s="253">
+        <f>IF(OR(E5="",F5=""),"",NETWORKDAYS(E5,F5,Ref!$K$2:$K$42))</f>
+        <v/>
+      </c>
+      <c r="AE5" s="253">
+        <f>IF(IFERROR(VLOOKUP(D5,Controls!$A$61:$E$71,2,FALSE),"No")="Yes",1,0)</f>
+        <v/>
+      </c>
+      <c r="AF5" s="253">
+        <f>IF(IFERROR(VLOOKUP(D5,Controls!$A$61:$E$71,3,FALSE),"No")="Yes",1,0)</f>
+        <v/>
+      </c>
+      <c r="AG5" s="253">
+        <f>IF(IFERROR(VLOOKUP(D5,Controls!$A$61:$E$71,4,FALSE),"No")="Yes",1,0)</f>
+        <v/>
+      </c>
+      <c r="AH5" s="253">
+        <f>IF(AND(E5&lt;&gt;"",E5&gt;=Controls!$B$37,E5&lt;=Controls!$B$38),1,0)</f>
+        <v/>
+      </c>
+      <c r="AI5" s="254">
+        <f>Q5-N5</f>
+        <v/>
+      </c>
+      <c r="AJ5" s="254">
+        <f>IF(AE5=1,MAX(0,N5-Q5),0)</f>
+        <v/>
+      </c>
+      <c r="AK5" s="255">
+        <f>IFERROR(Q5/N5,"")</f>
+        <v/>
+      </c>
+      <c r="AL5" s="255">
+        <f>IF(V5="","",N5/V5)</f>
+        <v/>
+      </c>
+      <c r="AM5" s="253">
+        <f>IF(V5="",0,1)</f>
+        <v/>
+      </c>
+      <c r="AN5" s="253">
+        <f>IF(Q5&lt;=0,1,0)</f>
+        <v/>
+      </c>
+      <c r="AO5" s="253">
+        <f>IF(AE5=1,AD5,"")</f>
+        <v/>
+      </c>
+      <c r="AP5" s="253">
+        <f>IF(AND(AE5=0,AG5=1),AD5,"")</f>
+        <v/>
+      </c>
+      <c r="AQ5" s="253">
+        <f>IF(N5&lt;10000,"Under $10K",IF(N5&lt;20000,"$10-20K",IF(N5&lt;30000,"$20-30K",IF(N5&lt;50000,"$30-50K",IF(N5&lt;100000,"$50-100K","$100K+")))))</f>
+        <v/>
+      </c>
+      <c r="AR5" s="253">
+        <f>IF(M5&lt;=1.35,"1.35 and under",IF(M5&lt;=1.42,"1.36-1.42",IF(M5&lt;=1.45,"1.43-1.45",IF(M5&lt;1.49,"1.46-1.48",IF(M5&lt;=1.49,"1.49","Above 1.49")))))</f>
+        <v/>
+      </c>
+      <c r="AS5" s="253">
+        <f>IF(AB5="","",IF(AB5&lt;60,"Under 60",IF(AB5&lt;90,"60-89",IF(AB5&lt;120,"90-119",IF(AB5&lt;150,"120-149","150+")))))</f>
+        <v/>
+      </c>
+      <c r="AT5" s="253">
+        <f>IF(AL5="","No revenue data",IF(AL5&lt;0.15,"Under 0.15x",IF(AL5&lt;0.3,"0.15-0.30x",IF(AL5&lt;0.5,"0.30-0.50x",IF(AL5&lt;1,"0.50-1.00x","1.00x+")))))</f>
+        <v/>
+      </c>
+      <c r="AU5" s="253">
+        <f>IF(I5="","No SIC",IFERROR(VLOOKUP(I5,Ref!$A$2:$B$65,2,FALSE),"Unclassified"))</f>
+        <v/>
+      </c>
+      <c r="AV5" s="253">
+        <f>IF(E5="","",TEXT(E5,"YYYY")&amp;"-Q"&amp;ROUNDUP(MONTH(E5)/3,0))</f>
+        <v/>
+      </c>
+      <c r="AW5" s="253">
+        <f>IF(E5="","",TEXT(E5,"YYYY-MM"))</f>
+        <v/>
+      </c>
+      <c r="AX5" s="253">
+        <f>IF(E5="","",TEXT(E5,"YYYY"))</f>
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -12187,10 +12653,10 @@
           <t>In House Collection</t>
         </is>
       </c>
-      <c r="E6" s="249" t="n">
+      <c r="E6" s="250" t="n">
         <v>45768</v>
       </c>
-      <c r="F6" s="249" t="n">
+      <c r="F6" s="250" t="n">
         <v>45889</v>
       </c>
       <c r="G6" t="n">
@@ -12224,22 +12690,22 @@
       <c r="M6" t="n">
         <v>1.5</v>
       </c>
-      <c r="N6" s="250" t="n">
+      <c r="N6" s="251" t="n">
         <v>40000</v>
       </c>
-      <c r="O6" s="250" t="n">
+      <c r="O6" s="251" t="n">
         <v>4000</v>
       </c>
-      <c r="P6" s="250" t="n">
+      <c r="P6" s="251" t="n">
         <v>60000</v>
       </c>
-      <c r="Q6" s="250" t="n">
+      <c r="Q6" s="251" t="n">
         <v>20000</v>
       </c>
-      <c r="R6" s="250" t="n">
+      <c r="R6" s="251" t="n">
         <v>40000</v>
       </c>
-      <c r="S6" s="251" t="n">
+      <c r="S6" s="252" t="n">
         <v>0.333333333333333</v>
       </c>
       <c r="T6" t="n">
@@ -12251,11 +12717,115 @@
       <c r="V6" t="n">
         <v>80000</v>
       </c>
-      <c r="W6" s="251" t="n">
+      <c r="W6" s="252" t="n">
         <v>0.11</v>
       </c>
-      <c r="X6" s="249" t="n">
+      <c r="X6" s="250" t="n">
         <v>41182</v>
+      </c>
+      <c r="Y6" s="253">
+        <f>IF(T6="","",IF(T6&lt;12,"Months","Weeks"))</f>
+        <v/>
+      </c>
+      <c r="Z6" s="253">
+        <f>IF(Y6="","",IF(Y6="Months","Daily","Weekly"))</f>
+        <v/>
+      </c>
+      <c r="AA6" s="253">
+        <f>IF(T6="","",IF(Z6="Daily",T6*Controls!$B$29,T6))</f>
+        <v/>
+      </c>
+      <c r="AB6" s="253">
+        <f>IF(T6="","",IF(Z6="Daily",T6*Controls!$B$29,T6*5))</f>
+        <v/>
+      </c>
+      <c r="AC6" s="253">
+        <f>IF(OR(E6="",F6=""),"",F6-E6)</f>
+        <v/>
+      </c>
+      <c r="AD6" s="253">
+        <f>IF(OR(E6="",F6=""),"",NETWORKDAYS(E6,F6,Ref!$K$2:$K$42))</f>
+        <v/>
+      </c>
+      <c r="AE6" s="253">
+        <f>IF(IFERROR(VLOOKUP(D6,Controls!$A$61:$E$71,2,FALSE),"No")="Yes",1,0)</f>
+        <v/>
+      </c>
+      <c r="AF6" s="253">
+        <f>IF(IFERROR(VLOOKUP(D6,Controls!$A$61:$E$71,3,FALSE),"No")="Yes",1,0)</f>
+        <v/>
+      </c>
+      <c r="AG6" s="253">
+        <f>IF(IFERROR(VLOOKUP(D6,Controls!$A$61:$E$71,4,FALSE),"No")="Yes",1,0)</f>
+        <v/>
+      </c>
+      <c r="AH6" s="253">
+        <f>IF(AND(E6&lt;&gt;"",E6&gt;=Controls!$B$37,E6&lt;=Controls!$B$38),1,0)</f>
+        <v/>
+      </c>
+      <c r="AI6" s="254">
+        <f>Q6-N6</f>
+        <v/>
+      </c>
+      <c r="AJ6" s="254">
+        <f>IF(AE6=1,MAX(0,N6-Q6),0)</f>
+        <v/>
+      </c>
+      <c r="AK6" s="255">
+        <f>IFERROR(Q6/N6,"")</f>
+        <v/>
+      </c>
+      <c r="AL6" s="255">
+        <f>IF(V6="","",N6/V6)</f>
+        <v/>
+      </c>
+      <c r="AM6" s="253">
+        <f>IF(V6="",0,1)</f>
+        <v/>
+      </c>
+      <c r="AN6" s="253">
+        <f>IF(Q6&lt;=0,1,0)</f>
+        <v/>
+      </c>
+      <c r="AO6" s="253">
+        <f>IF(AE6=1,AD6,"")</f>
+        <v/>
+      </c>
+      <c r="AP6" s="253">
+        <f>IF(AND(AE6=0,AG6=1),AD6,"")</f>
+        <v/>
+      </c>
+      <c r="AQ6" s="253">
+        <f>IF(N6&lt;10000,"Under $10K",IF(N6&lt;20000,"$10-20K",IF(N6&lt;30000,"$20-30K",IF(N6&lt;50000,"$30-50K",IF(N6&lt;100000,"$50-100K","$100K+")))))</f>
+        <v/>
+      </c>
+      <c r="AR6" s="253">
+        <f>IF(M6&lt;=1.35,"1.35 and under",IF(M6&lt;=1.42,"1.36-1.42",IF(M6&lt;=1.45,"1.43-1.45",IF(M6&lt;1.49,"1.46-1.48",IF(M6&lt;=1.49,"1.49","Above 1.49")))))</f>
+        <v/>
+      </c>
+      <c r="AS6" s="253">
+        <f>IF(AB6="","",IF(AB6&lt;60,"Under 60",IF(AB6&lt;90,"60-89",IF(AB6&lt;120,"90-119",IF(AB6&lt;150,"120-149","150+")))))</f>
+        <v/>
+      </c>
+      <c r="AT6" s="253">
+        <f>IF(AL6="","No revenue data",IF(AL6&lt;0.15,"Under 0.15x",IF(AL6&lt;0.3,"0.15-0.30x",IF(AL6&lt;0.5,"0.30-0.50x",IF(AL6&lt;1,"0.50-1.00x","1.00x+")))))</f>
+        <v/>
+      </c>
+      <c r="AU6" s="253">
+        <f>IF(I6="","No SIC",IFERROR(VLOOKUP(I6,Ref!$A$2:$B$65,2,FALSE),"Unclassified"))</f>
+        <v/>
+      </c>
+      <c r="AV6" s="253">
+        <f>IF(E6="","",TEXT(E6,"YYYY")&amp;"-Q"&amp;ROUNDUP(MONTH(E6)/3,0))</f>
+        <v/>
+      </c>
+      <c r="AW6" s="253">
+        <f>IF(E6="","",TEXT(E6,"YYYY-MM"))</f>
+        <v/>
+      </c>
+      <c r="AX6" s="253">
+        <f>IF(E6="","",TEXT(E6,"YYYY"))</f>
+        <v/>
       </c>
     </row>
     <row r="7">
@@ -12279,10 +12849,10 @@
           <t>Written-Off</t>
         </is>
       </c>
-      <c r="E7" s="249" t="n">
+      <c r="E7" s="250" t="n">
         <v>45789</v>
       </c>
-      <c r="F7" s="249" t="n">
+      <c r="F7" s="250" t="n">
         <v>45973</v>
       </c>
       <c r="G7" t="n">
@@ -12316,22 +12886,22 @@
       <c r="M7" t="n">
         <v>1.5</v>
       </c>
-      <c r="N7" s="250" t="n">
+      <c r="N7" s="251" t="n">
         <v>10000</v>
       </c>
-      <c r="O7" s="250" t="n">
+      <c r="O7" s="251" t="n">
         <v>1000</v>
       </c>
-      <c r="P7" s="250" t="n">
+      <c r="P7" s="251" t="n">
         <v>15000</v>
       </c>
-      <c r="Q7" s="250" t="n">
+      <c r="Q7" s="251" t="n">
         <v>9500</v>
       </c>
-      <c r="R7" s="250" t="n">
+      <c r="R7" s="251" t="n">
         <v>5500</v>
       </c>
-      <c r="S7" s="251" t="n">
+      <c r="S7" s="252" t="n">
         <v>0.633333333333333</v>
       </c>
       <c r="T7" t="n">
@@ -12343,11 +12913,115 @@
       <c r="V7" t="n">
         <v>20000</v>
       </c>
-      <c r="W7" s="251" t="n">
+      <c r="W7" s="252" t="n">
         <v>0.14</v>
       </c>
-      <c r="X7" s="249" t="n">
+      <c r="X7" s="250" t="n">
         <v>43774</v>
+      </c>
+      <c r="Y7" s="253">
+        <f>IF(T7="","",IF(T7&lt;12,"Months","Weeks"))</f>
+        <v/>
+      </c>
+      <c r="Z7" s="253">
+        <f>IF(Y7="","",IF(Y7="Months","Daily","Weekly"))</f>
+        <v/>
+      </c>
+      <c r="AA7" s="253">
+        <f>IF(T7="","",IF(Z7="Daily",T7*Controls!$B$29,T7))</f>
+        <v/>
+      </c>
+      <c r="AB7" s="253">
+        <f>IF(T7="","",IF(Z7="Daily",T7*Controls!$B$29,T7*5))</f>
+        <v/>
+      </c>
+      <c r="AC7" s="253">
+        <f>IF(OR(E7="",F7=""),"",F7-E7)</f>
+        <v/>
+      </c>
+      <c r="AD7" s="253">
+        <f>IF(OR(E7="",F7=""),"",NETWORKDAYS(E7,F7,Ref!$K$2:$K$42))</f>
+        <v/>
+      </c>
+      <c r="AE7" s="253">
+        <f>IF(IFERROR(VLOOKUP(D7,Controls!$A$61:$E$71,2,FALSE),"No")="Yes",1,0)</f>
+        <v/>
+      </c>
+      <c r="AF7" s="253">
+        <f>IF(IFERROR(VLOOKUP(D7,Controls!$A$61:$E$71,3,FALSE),"No")="Yes",1,0)</f>
+        <v/>
+      </c>
+      <c r="AG7" s="253">
+        <f>IF(IFERROR(VLOOKUP(D7,Controls!$A$61:$E$71,4,FALSE),"No")="Yes",1,0)</f>
+        <v/>
+      </c>
+      <c r="AH7" s="253">
+        <f>IF(AND(E7&lt;&gt;"",E7&gt;=Controls!$B$37,E7&lt;=Controls!$B$38),1,0)</f>
+        <v/>
+      </c>
+      <c r="AI7" s="254">
+        <f>Q7-N7</f>
+        <v/>
+      </c>
+      <c r="AJ7" s="254">
+        <f>IF(AE7=1,MAX(0,N7-Q7),0)</f>
+        <v/>
+      </c>
+      <c r="AK7" s="255">
+        <f>IFERROR(Q7/N7,"")</f>
+        <v/>
+      </c>
+      <c r="AL7" s="255">
+        <f>IF(V7="","",N7/V7)</f>
+        <v/>
+      </c>
+      <c r="AM7" s="253">
+        <f>IF(V7="",0,1)</f>
+        <v/>
+      </c>
+      <c r="AN7" s="253">
+        <f>IF(Q7&lt;=0,1,0)</f>
+        <v/>
+      </c>
+      <c r="AO7" s="253">
+        <f>IF(AE7=1,AD7,"")</f>
+        <v/>
+      </c>
+      <c r="AP7" s="253">
+        <f>IF(AND(AE7=0,AG7=1),AD7,"")</f>
+        <v/>
+      </c>
+      <c r="AQ7" s="253">
+        <f>IF(N7&lt;10000,"Under $10K",IF(N7&lt;20000,"$10-20K",IF(N7&lt;30000,"$20-30K",IF(N7&lt;50000,"$30-50K",IF(N7&lt;100000,"$50-100K","$100K+")))))</f>
+        <v/>
+      </c>
+      <c r="AR7" s="253">
+        <f>IF(M7&lt;=1.35,"1.35 and under",IF(M7&lt;=1.42,"1.36-1.42",IF(M7&lt;=1.45,"1.43-1.45",IF(M7&lt;1.49,"1.46-1.48",IF(M7&lt;=1.49,"1.49","Above 1.49")))))</f>
+        <v/>
+      </c>
+      <c r="AS7" s="253">
+        <f>IF(AB7="","",IF(AB7&lt;60,"Under 60",IF(AB7&lt;90,"60-89",IF(AB7&lt;120,"90-119",IF(AB7&lt;150,"120-149","150+")))))</f>
+        <v/>
+      </c>
+      <c r="AT7" s="253">
+        <f>IF(AL7="","No revenue data",IF(AL7&lt;0.15,"Under 0.15x",IF(AL7&lt;0.3,"0.15-0.30x",IF(AL7&lt;0.5,"0.30-0.50x",IF(AL7&lt;1,"0.50-1.00x","1.00x+")))))</f>
+        <v/>
+      </c>
+      <c r="AU7" s="253">
+        <f>IF(I7="","No SIC",IFERROR(VLOOKUP(I7,Ref!$A$2:$B$65,2,FALSE),"Unclassified"))</f>
+        <v/>
+      </c>
+      <c r="AV7" s="253">
+        <f>IF(E7="","",TEXT(E7,"YYYY")&amp;"-Q"&amp;ROUNDUP(MONTH(E7)/3,0))</f>
+        <v/>
+      </c>
+      <c r="AW7" s="253">
+        <f>IF(E7="","",TEXT(E7,"YYYY-MM"))</f>
+        <v/>
+      </c>
+      <c r="AX7" s="253">
+        <f>IF(E7="","",TEXT(E7,"YYYY"))</f>
+        <v/>
       </c>
     </row>
     <row r="8">
@@ -12371,10 +13045,10 @@
           <t>Bankruptcy</t>
         </is>
       </c>
-      <c r="E8" s="249" t="n">
+      <c r="E8" s="250" t="n">
         <v>45826</v>
       </c>
-      <c r="F8" s="249" t="n">
+      <c r="F8" s="250" t="n">
         <v>45918</v>
       </c>
       <c r="G8" t="n">
@@ -12398,22 +13072,22 @@
       <c r="M8" t="n">
         <v>1.5</v>
       </c>
-      <c r="N8" s="250" t="n">
+      <c r="N8" s="251" t="n">
         <v>20000</v>
       </c>
-      <c r="O8" s="250" t="n">
+      <c r="O8" s="251" t="n">
         <v>2000</v>
       </c>
-      <c r="P8" s="250" t="n">
+      <c r="P8" s="251" t="n">
         <v>30000</v>
       </c>
-      <c r="Q8" s="250" t="n">
+      <c r="Q8" s="251" t="n">
         <v>0</v>
       </c>
-      <c r="R8" s="250" t="n">
+      <c r="R8" s="251" t="n">
         <v>30000</v>
       </c>
-      <c r="S8" s="251" t="n">
+      <c r="S8" s="252" t="n">
         <v>0</v>
       </c>
       <c r="T8" t="n">
@@ -12425,11 +13099,115 @@
       <c r="V8" t="n">
         <v>100000</v>
       </c>
-      <c r="W8" s="251" t="n">
+      <c r="W8" s="252" t="n">
         <v>0.1</v>
       </c>
-      <c r="X8" s="249" t="n">
+      <c r="X8" s="250" t="n">
         <v>44305</v>
+      </c>
+      <c r="Y8" s="253">
+        <f>IF(T8="","",IF(T8&lt;12,"Months","Weeks"))</f>
+        <v/>
+      </c>
+      <c r="Z8" s="253">
+        <f>IF(Y8="","",IF(Y8="Months","Daily","Weekly"))</f>
+        <v/>
+      </c>
+      <c r="AA8" s="253">
+        <f>IF(T8="","",IF(Z8="Daily",T8*Controls!$B$29,T8))</f>
+        <v/>
+      </c>
+      <c r="AB8" s="253">
+        <f>IF(T8="","",IF(Z8="Daily",T8*Controls!$B$29,T8*5))</f>
+        <v/>
+      </c>
+      <c r="AC8" s="253">
+        <f>IF(OR(E8="",F8=""),"",F8-E8)</f>
+        <v/>
+      </c>
+      <c r="AD8" s="253">
+        <f>IF(OR(E8="",F8=""),"",NETWORKDAYS(E8,F8,Ref!$K$2:$K$42))</f>
+        <v/>
+      </c>
+      <c r="AE8" s="253">
+        <f>IF(IFERROR(VLOOKUP(D8,Controls!$A$61:$E$71,2,FALSE),"No")="Yes",1,0)</f>
+        <v/>
+      </c>
+      <c r="AF8" s="253">
+        <f>IF(IFERROR(VLOOKUP(D8,Controls!$A$61:$E$71,3,FALSE),"No")="Yes",1,0)</f>
+        <v/>
+      </c>
+      <c r="AG8" s="253">
+        <f>IF(IFERROR(VLOOKUP(D8,Controls!$A$61:$E$71,4,FALSE),"No")="Yes",1,0)</f>
+        <v/>
+      </c>
+      <c r="AH8" s="253">
+        <f>IF(AND(E8&lt;&gt;"",E8&gt;=Controls!$B$37,E8&lt;=Controls!$B$38),1,0)</f>
+        <v/>
+      </c>
+      <c r="AI8" s="254">
+        <f>Q8-N8</f>
+        <v/>
+      </c>
+      <c r="AJ8" s="254">
+        <f>IF(AE8=1,MAX(0,N8-Q8),0)</f>
+        <v/>
+      </c>
+      <c r="AK8" s="255">
+        <f>IFERROR(Q8/N8,"")</f>
+        <v/>
+      </c>
+      <c r="AL8" s="255">
+        <f>IF(V8="","",N8/V8)</f>
+        <v/>
+      </c>
+      <c r="AM8" s="253">
+        <f>IF(V8="",0,1)</f>
+        <v/>
+      </c>
+      <c r="AN8" s="253">
+        <f>IF(Q8&lt;=0,1,0)</f>
+        <v/>
+      </c>
+      <c r="AO8" s="253">
+        <f>IF(AE8=1,AD8,"")</f>
+        <v/>
+      </c>
+      <c r="AP8" s="253">
+        <f>IF(AND(AE8=0,AG8=1),AD8,"")</f>
+        <v/>
+      </c>
+      <c r="AQ8" s="253">
+        <f>IF(N8&lt;10000,"Under $10K",IF(N8&lt;20000,"$10-20K",IF(N8&lt;30000,"$20-30K",IF(N8&lt;50000,"$30-50K",IF(N8&lt;100000,"$50-100K","$100K+")))))</f>
+        <v/>
+      </c>
+      <c r="AR8" s="253">
+        <f>IF(M8&lt;=1.35,"1.35 and under",IF(M8&lt;=1.42,"1.36-1.42",IF(M8&lt;=1.45,"1.43-1.45",IF(M8&lt;1.49,"1.46-1.48",IF(M8&lt;=1.49,"1.49","Above 1.49")))))</f>
+        <v/>
+      </c>
+      <c r="AS8" s="253">
+        <f>IF(AB8="","",IF(AB8&lt;60,"Under 60",IF(AB8&lt;90,"60-89",IF(AB8&lt;120,"90-119",IF(AB8&lt;150,"120-149","150+")))))</f>
+        <v/>
+      </c>
+      <c r="AT8" s="253">
+        <f>IF(AL8="","No revenue data",IF(AL8&lt;0.15,"Under 0.15x",IF(AL8&lt;0.3,"0.15-0.30x",IF(AL8&lt;0.5,"0.30-0.50x",IF(AL8&lt;1,"0.50-1.00x","1.00x+")))))</f>
+        <v/>
+      </c>
+      <c r="AU8" s="253">
+        <f>IF(I8="","No SIC",IFERROR(VLOOKUP(I8,Ref!$A$2:$B$65,2,FALSE),"Unclassified"))</f>
+        <v/>
+      </c>
+      <c r="AV8" s="253">
+        <f>IF(E8="","",TEXT(E8,"YYYY")&amp;"-Q"&amp;ROUNDUP(MONTH(E8)/3,0))</f>
+        <v/>
+      </c>
+      <c r="AW8" s="253">
+        <f>IF(E8="","",TEXT(E8,"YYYY-MM"))</f>
+        <v/>
+      </c>
+      <c r="AX8" s="253">
+        <f>IF(E8="","",TEXT(E8,"YYYY"))</f>
+        <v/>
       </c>
     </row>
     <row r="9">
@@ -12453,10 +13231,10 @@
           <t>Open</t>
         </is>
       </c>
-      <c r="E9" s="249" t="n">
+      <c r="E9" s="250" t="n">
         <v>46030</v>
       </c>
-      <c r="F9" s="249" t="n">
+      <c r="F9" s="250" t="n">
         <v>46237</v>
       </c>
       <c r="G9" t="n">
@@ -12490,22 +13268,22 @@
       <c r="M9" t="n">
         <v>1.5</v>
       </c>
-      <c r="N9" s="250" t="n">
+      <c r="N9" s="251" t="n">
         <v>50000</v>
       </c>
-      <c r="O9" s="250" t="n">
+      <c r="O9" s="251" t="n">
         <v>5000</v>
       </c>
-      <c r="P9" s="250" t="n">
+      <c r="P9" s="251" t="n">
         <v>75000</v>
       </c>
-      <c r="Q9" s="250" t="n">
+      <c r="Q9" s="251" t="n">
         <v>30000</v>
       </c>
-      <c r="R9" s="250" t="n">
+      <c r="R9" s="251" t="n">
         <v>45000</v>
       </c>
-      <c r="S9" s="251" t="n">
+      <c r="S9" s="252" t="n">
         <v>0.4</v>
       </c>
       <c r="T9" t="n">
@@ -12517,11 +13295,115 @@
       <c r="V9" t="n">
         <v>250000</v>
       </c>
-      <c r="W9" s="251" t="n">
+      <c r="W9" s="252" t="n">
         <v>0.08</v>
       </c>
-      <c r="X9" s="249" t="n">
+      <c r="X9" s="250" t="n">
         <v>40211</v>
+      </c>
+      <c r="Y9" s="253">
+        <f>IF(T9="","",IF(T9&lt;12,"Months","Weeks"))</f>
+        <v/>
+      </c>
+      <c r="Z9" s="253">
+        <f>IF(Y9="","",IF(Y9="Months","Daily","Weekly"))</f>
+        <v/>
+      </c>
+      <c r="AA9" s="253">
+        <f>IF(T9="","",IF(Z9="Daily",T9*Controls!$B$29,T9))</f>
+        <v/>
+      </c>
+      <c r="AB9" s="253">
+        <f>IF(T9="","",IF(Z9="Daily",T9*Controls!$B$29,T9*5))</f>
+        <v/>
+      </c>
+      <c r="AC9" s="253">
+        <f>IF(OR(E9="",F9=""),"",F9-E9)</f>
+        <v/>
+      </c>
+      <c r="AD9" s="253">
+        <f>IF(OR(E9="",F9=""),"",NETWORKDAYS(E9,F9,Ref!$K$2:$K$42))</f>
+        <v/>
+      </c>
+      <c r="AE9" s="253">
+        <f>IF(IFERROR(VLOOKUP(D9,Controls!$A$61:$E$71,2,FALSE),"No")="Yes",1,0)</f>
+        <v/>
+      </c>
+      <c r="AF9" s="253">
+        <f>IF(IFERROR(VLOOKUP(D9,Controls!$A$61:$E$71,3,FALSE),"No")="Yes",1,0)</f>
+        <v/>
+      </c>
+      <c r="AG9" s="253">
+        <f>IF(IFERROR(VLOOKUP(D9,Controls!$A$61:$E$71,4,FALSE),"No")="Yes",1,0)</f>
+        <v/>
+      </c>
+      <c r="AH9" s="253">
+        <f>IF(AND(E9&lt;&gt;"",E9&gt;=Controls!$B$37,E9&lt;=Controls!$B$38),1,0)</f>
+        <v/>
+      </c>
+      <c r="AI9" s="254">
+        <f>Q9-N9</f>
+        <v/>
+      </c>
+      <c r="AJ9" s="254">
+        <f>IF(AE9=1,MAX(0,N9-Q9),0)</f>
+        <v/>
+      </c>
+      <c r="AK9" s="255">
+        <f>IFERROR(Q9/N9,"")</f>
+        <v/>
+      </c>
+      <c r="AL9" s="255">
+        <f>IF(V9="","",N9/V9)</f>
+        <v/>
+      </c>
+      <c r="AM9" s="253">
+        <f>IF(V9="",0,1)</f>
+        <v/>
+      </c>
+      <c r="AN9" s="253">
+        <f>IF(Q9&lt;=0,1,0)</f>
+        <v/>
+      </c>
+      <c r="AO9" s="253">
+        <f>IF(AE9=1,AD9,"")</f>
+        <v/>
+      </c>
+      <c r="AP9" s="253">
+        <f>IF(AND(AE9=0,AG9=1),AD9,"")</f>
+        <v/>
+      </c>
+      <c r="AQ9" s="253">
+        <f>IF(N9&lt;10000,"Under $10K",IF(N9&lt;20000,"$10-20K",IF(N9&lt;30000,"$20-30K",IF(N9&lt;50000,"$30-50K",IF(N9&lt;100000,"$50-100K","$100K+")))))</f>
+        <v/>
+      </c>
+      <c r="AR9" s="253">
+        <f>IF(M9&lt;=1.35,"1.35 and under",IF(M9&lt;=1.42,"1.36-1.42",IF(M9&lt;=1.45,"1.43-1.45",IF(M9&lt;1.49,"1.46-1.48",IF(M9&lt;=1.49,"1.49","Above 1.49")))))</f>
+        <v/>
+      </c>
+      <c r="AS9" s="253">
+        <f>IF(AB9="","",IF(AB9&lt;60,"Under 60",IF(AB9&lt;90,"60-89",IF(AB9&lt;120,"90-119",IF(AB9&lt;150,"120-149","150+")))))</f>
+        <v/>
+      </c>
+      <c r="AT9" s="253">
+        <f>IF(AL9="","No revenue data",IF(AL9&lt;0.15,"Under 0.15x",IF(AL9&lt;0.3,"0.15-0.30x",IF(AL9&lt;0.5,"0.30-0.50x",IF(AL9&lt;1,"0.50-1.00x","1.00x+")))))</f>
+        <v/>
+      </c>
+      <c r="AU9" s="253">
+        <f>IF(I9="","No SIC",IFERROR(VLOOKUP(I9,Ref!$A$2:$B$65,2,FALSE),"Unclassified"))</f>
+        <v/>
+      </c>
+      <c r="AV9" s="253">
+        <f>IF(E9="","",TEXT(E9,"YYYY")&amp;"-Q"&amp;ROUNDUP(MONTH(E9)/3,0))</f>
+        <v/>
+      </c>
+      <c r="AW9" s="253">
+        <f>IF(E9="","",TEXT(E9,"YYYY-MM"))</f>
+        <v/>
+      </c>
+      <c r="AX9" s="253">
+        <f>IF(E9="","",TEXT(E9,"YYYY"))</f>
+        <v/>
       </c>
     </row>
     <row r="10">
@@ -12545,10 +13427,10 @@
           <t>Closed/NSF Unpaid</t>
         </is>
       </c>
-      <c r="E10" s="249" t="n">
+      <c r="E10" s="250" t="n">
         <v>45852</v>
       </c>
-      <c r="F10" s="249" t="n">
+      <c r="F10" s="250" t="n">
         <v>46006</v>
       </c>
       <c r="G10" t="n">
@@ -12582,22 +13464,22 @@
       <c r="M10" t="n">
         <v>1.5</v>
       </c>
-      <c r="N10" s="250" t="n">
+      <c r="N10" s="251" t="n">
         <v>20000</v>
       </c>
-      <c r="O10" s="250" t="n">
+      <c r="O10" s="251" t="n">
         <v>2000</v>
       </c>
-      <c r="P10" s="250" t="n">
+      <c r="P10" s="251" t="n">
         <v>30000</v>
       </c>
-      <c r="Q10" s="250" t="n">
+      <c r="Q10" s="251" t="n">
         <v>30000</v>
       </c>
-      <c r="R10" s="250" t="n">
+      <c r="R10" s="251" t="n">
         <v>0</v>
       </c>
-      <c r="S10" s="251" t="n">
+      <c r="S10" s="252" t="n">
         <v>1</v>
       </c>
       <c r="T10" t="n">
@@ -12606,17 +13488,121 @@
       <c r="U10" t="n">
         <v>11</v>
       </c>
-      <c r="W10" s="251" t="n">
+      <c r="W10" s="252" t="n">
         <v>0.13</v>
       </c>
-      <c r="X10" s="249" t="n">
+      <c r="X10" s="250" t="n">
         <v>44781</v>
+      </c>
+      <c r="Y10" s="253">
+        <f>IF(T10="","",IF(T10&lt;12,"Months","Weeks"))</f>
+        <v/>
+      </c>
+      <c r="Z10" s="253">
+        <f>IF(Y10="","",IF(Y10="Months","Daily","Weekly"))</f>
+        <v/>
+      </c>
+      <c r="AA10" s="253">
+        <f>IF(T10="","",IF(Z10="Daily",T10*Controls!$B$29,T10))</f>
+        <v/>
+      </c>
+      <c r="AB10" s="253">
+        <f>IF(T10="","",IF(Z10="Daily",T10*Controls!$B$29,T10*5))</f>
+        <v/>
+      </c>
+      <c r="AC10" s="253">
+        <f>IF(OR(E10="",F10=""),"",F10-E10)</f>
+        <v/>
+      </c>
+      <c r="AD10" s="253">
+        <f>IF(OR(E10="",F10=""),"",NETWORKDAYS(E10,F10,Ref!$K$2:$K$42))</f>
+        <v/>
+      </c>
+      <c r="AE10" s="253">
+        <f>IF(IFERROR(VLOOKUP(D10,Controls!$A$61:$E$71,2,FALSE),"No")="Yes",1,0)</f>
+        <v/>
+      </c>
+      <c r="AF10" s="253">
+        <f>IF(IFERROR(VLOOKUP(D10,Controls!$A$61:$E$71,3,FALSE),"No")="Yes",1,0)</f>
+        <v/>
+      </c>
+      <c r="AG10" s="253">
+        <f>IF(IFERROR(VLOOKUP(D10,Controls!$A$61:$E$71,4,FALSE),"No")="Yes",1,0)</f>
+        <v/>
+      </c>
+      <c r="AH10" s="253">
+        <f>IF(AND(E10&lt;&gt;"",E10&gt;=Controls!$B$37,E10&lt;=Controls!$B$38),1,0)</f>
+        <v/>
+      </c>
+      <c r="AI10" s="254">
+        <f>Q10-N10</f>
+        <v/>
+      </c>
+      <c r="AJ10" s="254">
+        <f>IF(AE10=1,MAX(0,N10-Q10),0)</f>
+        <v/>
+      </c>
+      <c r="AK10" s="255">
+        <f>IFERROR(Q10/N10,"")</f>
+        <v/>
+      </c>
+      <c r="AL10" s="255">
+        <f>IF(V10="","",N10/V10)</f>
+        <v/>
+      </c>
+      <c r="AM10" s="253">
+        <f>IF(V10="",0,1)</f>
+        <v/>
+      </c>
+      <c r="AN10" s="253">
+        <f>IF(Q10&lt;=0,1,0)</f>
+        <v/>
+      </c>
+      <c r="AO10" s="253">
+        <f>IF(AE10=1,AD10,"")</f>
+        <v/>
+      </c>
+      <c r="AP10" s="253">
+        <f>IF(AND(AE10=0,AG10=1),AD10,"")</f>
+        <v/>
+      </c>
+      <c r="AQ10" s="253">
+        <f>IF(N10&lt;10000,"Under $10K",IF(N10&lt;20000,"$10-20K",IF(N10&lt;30000,"$20-30K",IF(N10&lt;50000,"$30-50K",IF(N10&lt;100000,"$50-100K","$100K+")))))</f>
+        <v/>
+      </c>
+      <c r="AR10" s="253">
+        <f>IF(M10&lt;=1.35,"1.35 and under",IF(M10&lt;=1.42,"1.36-1.42",IF(M10&lt;=1.45,"1.43-1.45",IF(M10&lt;1.49,"1.46-1.48",IF(M10&lt;=1.49,"1.49","Above 1.49")))))</f>
+        <v/>
+      </c>
+      <c r="AS10" s="253">
+        <f>IF(AB10="","",IF(AB10&lt;60,"Under 60",IF(AB10&lt;90,"60-89",IF(AB10&lt;120,"90-119",IF(AB10&lt;150,"120-149","150+")))))</f>
+        <v/>
+      </c>
+      <c r="AT10" s="253">
+        <f>IF(AL10="","No revenue data",IF(AL10&lt;0.15,"Under 0.15x",IF(AL10&lt;0.3,"0.15-0.30x",IF(AL10&lt;0.5,"0.30-0.50x",IF(AL10&lt;1,"0.50-1.00x","1.00x+")))))</f>
+        <v/>
+      </c>
+      <c r="AU10" s="253">
+        <f>IF(I10="","No SIC",IFERROR(VLOOKUP(I10,Ref!$A$2:$B$65,2,FALSE),"Unclassified"))</f>
+        <v/>
+      </c>
+      <c r="AV10" s="253">
+        <f>IF(E10="","",TEXT(E10,"YYYY")&amp;"-Q"&amp;ROUNDUP(MONTH(E10)/3,0))</f>
+        <v/>
+      </c>
+      <c r="AW10" s="253">
+        <f>IF(E10="","",TEXT(E10,"YYYY-MM"))</f>
+        <v/>
+      </c>
+      <c r="AX10" s="253">
+        <f>IF(E10="","",TEXT(E10,"YYYY"))</f>
+        <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="236" t="inlineStr">
         <is>
-          <t>8 synthetic sample deals from Copy_of_House_Book_Analytics.xlsx. The build replaces these with the full CRM export (1,067 rows, same column order). Helper columns become formulas filled down every row.</t>
+          <t>8 synthetic sample deals from Copy_of_House_Book_Analytics.xlsx. Green headers = helper columns carried over from House Book Analytics with their formulas live (re-pointed to this workbook's Controls and Ref). Dark headers = new columns for the matching engine, outlined only. The build replaces the samples with the full CRM export (1,067 rows) and fills every helper column down.</t>
         </is>
       </c>
     </row>
@@ -12705,13 +13691,13 @@
           <t>Total LVG (all debt / rev)</t>
         </is>
       </c>
-      <c r="B5" s="252" t="n">
+      <c r="B5" s="256" t="n">
         <v>0.3</v>
       </c>
-      <c r="C5" s="252" t="n">
+      <c r="C5" s="256" t="n">
         <v>0.45</v>
       </c>
-      <c r="D5" s="252" t="n">
+      <c r="D5" s="256" t="n">
         <v>0.55</v>
       </c>
       <c r="E5" s="245" t="inlineStr">
@@ -12731,13 +13717,13 @@
           <t>New holdback SP%</t>
         </is>
       </c>
-      <c r="B6" s="252" t="n">
+      <c r="B6" s="256" t="n">
         <v>0.18</v>
       </c>
-      <c r="C6" s="252" t="n">
+      <c r="C6" s="256" t="n">
         <v>0.25</v>
       </c>
-      <c r="D6" s="252" t="n">
+      <c r="D6" s="256" t="n">
         <v>0.35</v>
       </c>
       <c r="E6" s="245" t="inlineStr">
@@ -12753,13 +13739,13 @@
           <t>Daily debt / balance</t>
         </is>
       </c>
-      <c r="B7" s="252" t="n">
+      <c r="B7" s="256" t="n">
         <v>0.18</v>
       </c>
-      <c r="C7" s="252" t="n">
+      <c r="C7" s="256" t="n">
         <v>0.3</v>
       </c>
-      <c r="D7" s="252" t="n">
+      <c r="D7" s="256" t="n">
         <v>0.35</v>
       </c>
       <c r="E7" s="245" t="inlineStr">
@@ -12775,13 +13761,13 @@
           <t>Fund / revenue</t>
         </is>
       </c>
-      <c r="B8" s="253" t="n">
+      <c r="B8" s="257" t="n">
         <v>0.6</v>
       </c>
-      <c r="C8" s="253" t="n">
+      <c r="C8" s="257" t="n">
         <v>0.9</v>
       </c>
-      <c r="D8" s="253" t="n">
+      <c r="D8" s="257" t="n">
         <v>1.25</v>
       </c>
       <c r="E8" s="245" t="inlineStr">
@@ -12797,13 +13783,13 @@
           <t># positions (incl. new)</t>
         </is>
       </c>
-      <c r="B9" s="254" t="n">
+      <c r="B9" s="258" t="n">
         <v>2</v>
       </c>
-      <c r="C9" s="254" t="n">
+      <c r="C9" s="258" t="n">
         <v>5</v>
       </c>
-      <c r="D9" s="254" t="n">
+      <c r="D9" s="258" t="n">
         <v>6</v>
       </c>
       <c r="E9" s="245" t="inlineStr">
@@ -12819,13 +13805,13 @@
           <t>Revenue trend (avg MoM)</t>
         </is>
       </c>
-      <c r="B10" s="252" t="n">
+      <c r="B10" s="256" t="n">
         <v>-0.05</v>
       </c>
-      <c r="C10" s="252" t="n">
+      <c r="C10" s="256" t="n">
         <v>-0.15</v>
       </c>
-      <c r="D10" s="252" t="n">
+      <c r="D10" s="256" t="n">
         <v>-0.3</v>
       </c>
       <c r="E10" s="245" t="inlineStr">
@@ -12841,13 +13827,13 @@
           <t>Neg days + NSFs (total)</t>
         </is>
       </c>
-      <c r="B11" s="254" t="n">
+      <c r="B11" s="258" t="n">
         <v>1</v>
       </c>
-      <c r="C11" s="254" t="n">
+      <c r="C11" s="258" t="n">
         <v>6</v>
       </c>
-      <c r="D11" s="254" t="n">
+      <c r="D11" s="258" t="n">
         <v>10</v>
       </c>
       <c r="E11" s="245" t="inlineStr">
@@ -12867,13 +13853,13 @@
           <t>Credit score (FICO)  - NEW</t>
         </is>
       </c>
-      <c r="B12" s="254" t="n">
+      <c r="B12" s="258" t="n">
         <v>650</v>
       </c>
-      <c r="C12" s="254" t="n">
+      <c r="C12" s="258" t="n">
         <v>630</v>
       </c>
-      <c r="D12" s="254" t="n">
+      <c r="D12" s="258" t="n">
         <v>0</v>
       </c>
       <c r="E12" s="245" t="inlineStr">
@@ -12893,7 +13879,7 @@
           <t>Decline if red flags (RED + KNOCKOUT) &gt;=</t>
         </is>
       </c>
-      <c r="B13" s="254" t="n">
+      <c r="B13" s="258" t="n">
         <v>2</v>
       </c>
     </row>
@@ -12903,7 +13889,7 @@
           <t>Minimum fund $</t>
         </is>
       </c>
-      <c r="B14" s="255" t="n">
+      <c r="B14" s="259" t="n">
         <v>10000</v>
       </c>
       <c r="H14" s="236" t="inlineStr">
@@ -12918,7 +13904,7 @@
           <t>Underwriting fee %</t>
         </is>
       </c>
-      <c r="B15" s="256" t="n">
+      <c r="B15" s="260" t="n">
         <v>0.05</v>
       </c>
     </row>
@@ -12956,13 +13942,13 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="257" t="n">
+      <c r="A19" s="261" t="n">
         <v>0</v>
       </c>
-      <c r="B19" s="254" t="n">
+      <c r="B19" s="258" t="n">
         <v>100</v>
       </c>
-      <c r="C19" s="253" t="n">
+      <c r="C19" s="257" t="n">
         <v>1.49</v>
       </c>
       <c r="H19" s="236" t="inlineStr">
@@ -12972,35 +13958,35 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="257" t="n">
+      <c r="A20" s="261" t="n">
         <v>5</v>
       </c>
-      <c r="B20" s="254" t="n">
+      <c r="B20" s="258" t="n">
         <v>130</v>
       </c>
-      <c r="C20" s="253" t="n">
+      <c r="C20" s="257" t="n">
         <v>1.45</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="257" t="n">
+      <c r="A21" s="261" t="n">
         <v>6</v>
       </c>
-      <c r="B21" s="254" t="n">
+      <c r="B21" s="258" t="n">
         <v>150</v>
       </c>
-      <c r="C21" s="253" t="n">
+      <c r="C21" s="257" t="n">
         <v>1.45</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="257" t="n">
+      <c r="A22" s="261" t="n">
         <v>7</v>
       </c>
-      <c r="B22" s="254" t="n">
+      <c r="B22" s="258" t="n">
         <v>195</v>
       </c>
-      <c r="C22" s="253" t="n">
+      <c r="C22" s="257" t="n">
         <v>1.4</v>
       </c>
     </row>
@@ -13010,7 +13996,7 @@
           <t>Max term (months)</t>
         </is>
       </c>
-      <c r="B23" s="254" t="n">
+      <c r="B23" s="258" t="n">
         <v>9</v>
       </c>
     </row>
@@ -13020,13 +14006,13 @@
           <t>Approved factor tiers</t>
         </is>
       </c>
-      <c r="B24" s="253" t="n">
+      <c r="B24" s="257" t="n">
         <v>1.4</v>
       </c>
-      <c r="C24" s="253" t="n">
+      <c r="C24" s="257" t="n">
         <v>1.45</v>
       </c>
-      <c r="D24" s="253" t="n">
+      <c r="D24" s="257" t="n">
         <v>1.49</v>
       </c>
       <c r="H24" s="236" t="inlineStr">
@@ -13041,13 +14027,13 @@
           <t>Tier cut-offs (7-point scale): Strong / Solid / Moderate</t>
         </is>
       </c>
-      <c r="B25" s="257" t="n">
+      <c r="B25" s="261" t="n">
         <v>6.5</v>
       </c>
-      <c r="C25" s="257" t="n">
+      <c r="C25" s="261" t="n">
         <v>5</v>
       </c>
-      <c r="D25" s="257" t="n">
+      <c r="D25" s="261" t="n">
         <v>3.5</v>
       </c>
       <c r="H25" s="236" t="inlineStr">
@@ -13069,7 +14055,7 @@
           <t>Weeks per month (ours)</t>
         </is>
       </c>
-      <c r="B28" s="258" t="n">
+      <c r="B28" s="262" t="n">
         <v>4.331</v>
       </c>
       <c r="H28" s="236" t="inlineStr">
@@ -13084,7 +14070,7 @@
           <t>Business days per month (ours)</t>
         </is>
       </c>
-      <c r="B29" s="258" t="n">
+      <c r="B29" s="262" t="n">
         <v>21.655</v>
       </c>
       <c r="H29" s="236" t="inlineStr">
@@ -13099,7 +14085,7 @@
           <t>MoneyBadger weeks / month</t>
         </is>
       </c>
-      <c r="B30" s="254" t="n">
+      <c r="B30" s="258" t="n">
         <v>4</v>
       </c>
       <c r="H30" s="236" t="inlineStr"/>
@@ -13110,7 +14096,7 @@
           <t>MoneyBadger business days / month</t>
         </is>
       </c>
-      <c r="B31" s="254" t="n">
+      <c r="B31" s="258" t="n">
         <v>21</v>
       </c>
       <c r="H31" s="236" t="inlineStr"/>
@@ -13121,7 +14107,7 @@
           <t>Calendar days / month</t>
         </is>
       </c>
-      <c r="B32" s="259" t="n">
+      <c r="B32" s="263" t="n">
         <v>30.4375</v>
       </c>
       <c r="H32" s="236" t="inlineStr"/>
@@ -13132,7 +14118,7 @@
           <t>Assumed factor on existing positions</t>
         </is>
       </c>
-      <c r="B33" s="253" t="n">
+      <c r="B33" s="257" t="n">
         <v>1.45</v>
       </c>
       <c r="H33" s="236" t="inlineStr"/>
@@ -13150,7 +14136,7 @@
           <t>As-of date for seasoning (date of the CRM export)</t>
         </is>
       </c>
-      <c r="B36" s="260" t="n">
+      <c r="B36" s="264" t="n">
         <v>46259</v>
       </c>
       <c r="H36" s="236" t="inlineStr">
@@ -13165,7 +14151,7 @@
           <t>Window: funded on or after</t>
         </is>
       </c>
-      <c r="B37" s="260" t="n">
+      <c r="B37" s="264" t="n">
         <v>45597</v>
       </c>
       <c r="H37" s="236" t="inlineStr"/>
@@ -13176,7 +14162,7 @@
           <t>Window: funded on or before</t>
         </is>
       </c>
-      <c r="B38" s="260" t="n">
+      <c r="B38" s="264" t="n">
         <v>46259</v>
       </c>
       <c r="H38" s="236" t="inlineStr">
@@ -13191,7 +14177,7 @@
           <t>Seasoning multiple (age &gt;= multiple x contracted term)</t>
         </is>
       </c>
-      <c r="B39" s="253" t="n">
+      <c r="B39" s="257" t="n">
         <v>1.25</v>
       </c>
       <c r="H39" s="236" t="inlineStr">
@@ -13206,7 +14192,7 @@
           <t>Minimum seasoned deals for a cohort to be PRIMARY</t>
         </is>
       </c>
-      <c r="B40" s="254" t="n">
+      <c r="B40" s="258" t="n">
         <v>10</v>
       </c>
       <c r="H40" s="236" t="inlineStr"/>
@@ -13217,7 +14203,7 @@
           <t>Minimum seasoned funded $ for a cohort to be PRIMARY</t>
         </is>
       </c>
-      <c r="B41" s="255" t="n">
+      <c r="B41" s="259" t="n">
         <v>150000</v>
       </c>
       <c r="H41" s="236" t="inlineStr"/>
@@ -13228,7 +14214,7 @@
           <t>Credibility constant K</t>
         </is>
       </c>
-      <c r="B42" s="254" t="n">
+      <c r="B42" s="258" t="n">
         <v>30</v>
       </c>
       <c r="H42" s="236" t="inlineStr">
@@ -13243,7 +14229,7 @@
           <t>Max open share for "seasoned-enough"</t>
         </is>
       </c>
-      <c r="B43" s="256" t="n">
+      <c r="B43" s="260" t="n">
         <v>0.15</v>
       </c>
       <c r="H43" s="236" t="inlineStr"/>
@@ -13254,7 +14240,7 @@
           <t>High confidence: min Z</t>
         </is>
       </c>
-      <c r="B44" s="253" t="n">
+      <c r="B44" s="257" t="n">
         <v>0.6</v>
       </c>
       <c r="H44" s="236" t="inlineStr"/>
@@ -13265,7 +14251,7 @@
           <t>Medium confidence: min Z</t>
         </is>
       </c>
-      <c r="B45" s="253" t="n">
+      <c r="B45" s="257" t="n">
         <v>0.3</v>
       </c>
       <c r="H45" s="236" t="inlineStr"/>
@@ -13276,7 +14262,7 @@
           <t>Low confidence: max steps from Neutral</t>
         </is>
       </c>
-      <c r="B46" s="254" t="n">
+      <c r="B46" s="258" t="n">
         <v>1</v>
       </c>
       <c r="H46" s="236" t="inlineStr">
@@ -13291,7 +14277,7 @@
           <t>Minimum seasoned deals before a rate is shown</t>
         </is>
       </c>
-      <c r="B47" s="254" t="n">
+      <c r="B47" s="258" t="n">
         <v>5</v>
       </c>
       <c r="H47" s="236" t="inlineStr"/>
@@ -13346,7 +14332,7 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="253" t="n">
+      <c r="A51" s="257" t="n">
         <v>0.6</v>
       </c>
       <c r="B51" s="240" t="inlineStr">
@@ -13354,7 +14340,7 @@
           <t>Strong positive</t>
         </is>
       </c>
-      <c r="C51" s="253" t="n">
+      <c r="C51" s="257" t="n">
         <v>1</v>
       </c>
       <c r="D51" s="241" t="n">
@@ -13380,7 +14366,7 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="253" t="n">
+      <c r="A52" s="257" t="n">
         <v>0.85</v>
       </c>
       <c r="B52" s="240" t="inlineStr">
@@ -13388,7 +14374,7 @@
           <t>Mild positive</t>
         </is>
       </c>
-      <c r="C52" s="253" t="n">
+      <c r="C52" s="257" t="n">
         <v>0.95</v>
       </c>
       <c r="D52" s="241" t="n">
@@ -13410,7 +14396,7 @@
       <c r="H52" s="236" t="inlineStr"/>
     </row>
     <row r="53">
-      <c r="A53" s="253" t="n">
+      <c r="A53" s="257" t="n">
         <v>1.15</v>
       </c>
       <c r="B53" s="240" t="inlineStr">
@@ -13418,7 +14404,7 @@
           <t>Neutral</t>
         </is>
       </c>
-      <c r="C53" s="253" t="n">
+      <c r="C53" s="257" t="n">
         <v>0.9</v>
       </c>
       <c r="D53" s="241" t="n">
@@ -13444,7 +14430,7 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="253" t="n">
+      <c r="A54" s="257" t="n">
         <v>1.4</v>
       </c>
       <c r="B54" s="240" t="inlineStr">
@@ -13452,7 +14438,7 @@
           <t>Mild negative</t>
         </is>
       </c>
-      <c r="C54" s="253" t="n">
+      <c r="C54" s="257" t="n">
         <v>0.8</v>
       </c>
       <c r="D54" s="241" t="n">
@@ -13474,7 +14460,7 @@
       <c r="H54" s="236" t="inlineStr"/>
     </row>
     <row r="55">
-      <c r="A55" s="253" t="n">
+      <c r="A55" s="257" t="n">
         <v>1.75</v>
       </c>
       <c r="B55" s="240" t="inlineStr">
@@ -13482,7 +14468,7 @@
           <t>Negative</t>
         </is>
       </c>
-      <c r="C55" s="253" t="n">
+      <c r="C55" s="257" t="n">
         <v>0.7</v>
       </c>
       <c r="D55" s="241" t="n">
@@ -13508,7 +14494,7 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="253" t="n">
+      <c r="A56" s="257" t="n">
         <v>999</v>
       </c>
       <c r="B56" s="240" t="inlineStr">
@@ -13516,7 +14502,7 @@
           <t>Severe</t>
         </is>
       </c>
-      <c r="C56" s="253" t="n">
+      <c r="C56" s="257" t="n">
         <v>0.55</v>
       </c>
       <c r="D56" s="241" t="n">
@@ -13959,7 +14945,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="C79" s="254" t="n">
+      <c r="C79" s="258" t="n">
         <v>4</v>
       </c>
       <c r="H79" s="236" t="inlineStr">
@@ -13979,7 +14965,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="C80" s="254" t="n">
+      <c r="C80" s="258" t="n">
         <v>3</v>
       </c>
       <c r="H80" s="236" t="inlineStr">
@@ -14339,7 +15325,7 @@
       </c>
     </row>
     <row r="5" ht="45" customHeight="1" s="230">
-      <c r="B5" s="261" t="inlineStr">
+      <c r="B5" s="265" t="inlineStr">
         <is>
           <t>Bank data, avg balance, new/renewal, ISO, industry, state, credit score, requested offer, factor is an approved tier</t>
         </is>
@@ -14363,7 +15349,7 @@
       </c>
     </row>
     <row r="7" ht="45" customHeight="1" s="230">
-      <c r="B7" s="261" t="inlineStr">
+      <c r="B7" s="265" t="inlineStr">
         <is>
           <t>Error count on Deal / Historical Data / Historical Score / Offer Engine / Decision Summary</t>
         </is>
@@ -14387,7 +15373,7 @@
       </c>
     </row>
     <row r="9" ht="45" customHeight="1" s="230">
-      <c r="B9" s="261" t="inlineStr">
+      <c r="B9" s="265" t="inlineStr">
         <is>
           <t>Adjusted fund &lt;= cash-flow max; adjusted daily &lt;= max daily; no offer-side red at adjusted offer; merchant knockouts untouched</t>
         </is>
@@ -14411,7 +15397,7 @@
       </c>
     </row>
     <row r="11" ht="45" customHeight="1" s="230">
-      <c r="B11" s="261" t="inlineStr">
+      <c r="B11" s="265" t="inlineStr">
         <is>
           <t>Primary cohort met the minimums; seasoned-enough; Z at least Medium; no ISO-vs-industry conflict; tighter tiers skipped; state informational</t>
         </is>
@@ -14435,7 +15421,7 @@
       </c>
     </row>
     <row r="13" ht="45" customHeight="1" s="230">
-      <c r="B13" s="261" t="inlineStr">
+      <c r="B13" s="265" t="inlineStr">
         <is>
           <t>Deals loaded; unmapped statuses; no revenue; no ISO / state / SIC; never-paid; Open but fully paid; Open past 1.5x term; weekly term &gt; 39 weeks; position-3 concentration; Lowered Payments treatment; Written-Off collected most of payback</t>
         </is>
@@ -14459,7 +15445,7 @@
       </c>
     </row>
     <row r="15" ht="45" customHeight="1" s="230">
-      <c r="B15" s="261" t="inlineStr">
+      <c r="B15" s="265" t="inlineStr">
         <is>
           <t>Total funded $34,481,626; collected $27,438,510; principal lost $5,270,163; lost rate 15.3%; payback = advance x factor; seasoned-book size; tier-7 funded = in-window seasoned funded; comparable list count = cohort matches</t>
         </is>

</xml_diff>